<commit_message>
7 Day Kitchens: add Service Pages tab to keyword workbook
Service-page architecture (TJ addendum): core kitchen, Kitchen+X combos,
segment + component pages, suburb service-area pages. Real SEMrush US volumes.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/7-day-kitchens/keyword-research.xlsx
+++ b/decks/7-day-kitchens/keyword-research.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Article Plan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Keyword Universe" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Excluded" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Read Me" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Service Pages" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Keyword Universe" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Excluded" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Read Me" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +33,9 @@
       <b val="1"/>
       <color rgb="00F5EFE6"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -52,7 +56,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -94,6 +98,16 @@
         <fgColor rgb="00162f41"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFECE6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -107,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -125,13 +139,28 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5123,6 +5152,1216 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="66" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Service Page</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Primary Keyword</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>US Vol</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>KD</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Intent</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Why / Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Core Kitchen</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Kitchen Remodeling</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>kitchen remodeling charlotte</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H2" s="10" t="inlineStr">
+        <is>
+          <t>Have — expand</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Flagship money page. Strengthen with schema + internal links from the blog.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Core Kitchen</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Kitchen Design</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>kitchen design</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>22200</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <v>65</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>Have — expand</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Existing page. Design-led buyers; rank the local slice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Kitchen + X</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Kitchen + Bath Remodeling</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>kitchen and bath remodeling</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>4400</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>The anchor combo. Real demand + the 'get it all done at once' buyer Barry described.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kitchen + X</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Kitchen + Walk-in Pantry</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>walk in pantry</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>4400</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Low KD, strong demand. Premium add-on to a kitchen remodel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Small Kitchen Remodeling</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>small kitchen remodel</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>6600</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Easy win, high demand. Condo / townhome buyers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Luxury Kitchen Remodeling</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>luxury kitchen remodel</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Very low KD, matches your premium fixed-price positioning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Service Area</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Charlotte (hub)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>kitchen remodeling charlotte</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>Have</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Core geo page every suburb page links up to.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Service Area</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Waxhaw, NC</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>kitchen remodeling waxhaw nc</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>Have</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Existing service-area page. Map-pack + exact local intent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Service Area</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Matthews, NC</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>kitchen remodeling matthews nc</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Very winnable suburb (KD 4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Kitchen + X</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Kitchen + Scullery / Butler's Pantry</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>butlers pantry</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>9900</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>50</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Huge feature-research demand (scullery 18.1K, butler's pantry 9.9K). Premium differentiator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Kitchen + X</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Kitchen + Laundry Room</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>kitchen and laundry room</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>140</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Low direct search but a common combo; routes AI/Google to the right page (Onn's point).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Open-Concept Kitchen</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>open concept kitchen</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>1900</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Wall-removal / layout-change projects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Galley Kitchen Remodeling</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>galley kitchen remodel</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Layout-specific segment page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Custom Kitchen Cabinets</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>custom kitchen cabinets</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>8100</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>54</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>High-intent sub-service; part of every remodel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Kitchen Cabinet Refacing</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>kitchen cabinet refacing</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>6600</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Budget-tier service; you already rank ~#6 locally (GSC).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Service Area</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Marvin, NC</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>kitchen remodeling marvin nc</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Affluent suburb; you have a featured project there already.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Service Area</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Monroe, NC</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>kitchen remodeling monroe nc</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Union County.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Service Area</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Ballantyne</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>kitchen remodeling ballantyne</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Affluent South Charlotte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Kitchen + X</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Kitchen + Mudroom</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>kitchen and mudroom</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Intent-accuracy; supporting page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Custom Kitchens</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>custom kitchen</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F21" s="11" t="n">
+        <v>58</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Bespoke positioning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Kitchen Countertops</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>kitchen countertops</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>40500</v>
+      </c>
+      <c r="F22" s="11" t="n">
+        <v>58</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Massive demand; feature-as-service that funnels to full remodels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Kitchen Islands</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>kitchen island</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>90500</v>
+      </c>
+      <c r="F23" s="11" t="n">
+        <v>61</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Highest demand of all (90.5K); high KD. Feature page funneling to remodels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Kitchen Backsplash</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>kitchen backsplash</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>27100</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>High-demand feature page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Service Area</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Weddington, NC</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>kitchen remodeling weddington nc</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Expansion suburb.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Service Area</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Fort Mill, SC</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>kitchen remodeling fort mill sc</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>SC side of the metro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Service Area</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Huntersville / Mooresville / Belmont</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>kitchen remodeling &lt;suburb&gt; nc</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>North / west metro expansion pages.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5199,7 +6438,7 @@
       <c r="F2" s="5" t="n">
         <v>35</v>
       </c>
-      <c r="G2" s="9" t="inlineStr">
+      <c r="G2" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -5232,7 +6471,7 @@
       <c r="F3" s="5" t="n">
         <v>33</v>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="G3" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -5265,7 +6504,7 @@
       <c r="F4" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -5298,7 +6537,7 @@
       <c r="F5" s="5" t="n">
         <v>48</v>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="G5" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -5397,7 +6636,7 @@
       <c r="F8" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="G8" s="9" t="inlineStr">
+      <c r="G8" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -5430,7 +6669,7 @@
       <c r="F9" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="G9" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -5463,7 +6702,7 @@
       <c r="F10" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="G10" s="9" t="inlineStr">
+      <c r="G10" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -5496,7 +6735,7 @@
       <c r="F11" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="G11" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -5562,7 +6801,7 @@
       <c r="F13" s="5" t="n">
         <v>41</v>
       </c>
-      <c r="G13" s="9" t="inlineStr">
+      <c r="G13" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -5628,7 +6867,7 @@
       <c r="F15" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="G15" s="9" t="inlineStr">
+      <c r="G15" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -5661,7 +6900,7 @@
       <c r="F16" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="G16" s="9" t="inlineStr">
+      <c r="G16" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -5694,7 +6933,7 @@
       <c r="F17" s="5" t="n">
         <v>42</v>
       </c>
-      <c r="G17" s="9" t="inlineStr">
+      <c r="G17" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -5727,7 +6966,7 @@
       <c r="F18" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="G18" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -5793,7 +7032,7 @@
       <c r="F20" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="G20" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -5826,7 +7065,7 @@
       <c r="F21" s="5" t="n">
         <v>48</v>
       </c>
-      <c r="G21" s="9" t="inlineStr">
+      <c r="G21" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -5859,7 +7098,7 @@
       <c r="F22" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="G22" s="9" t="inlineStr">
+      <c r="G22" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -5892,7 +7131,7 @@
       <c r="F23" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="G23" s="9" t="inlineStr">
+      <c r="G23" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -5925,7 +7164,7 @@
       <c r="F24" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G24" s="9" t="inlineStr">
+      <c r="G24" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -5958,7 +7197,7 @@
       <c r="F25" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G25" s="9" t="inlineStr">
+      <c r="G25" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -5991,7 +7230,7 @@
       <c r="F26" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="G26" s="9" t="inlineStr">
+      <c r="G26" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -6057,7 +7296,7 @@
       <c r="F28" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="G28" s="9" t="inlineStr">
+      <c r="G28" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -6090,7 +7329,7 @@
       <c r="F29" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G29" s="9" t="inlineStr">
+      <c r="G29" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -6123,7 +7362,7 @@
       <c r="F30" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="G30" s="9" t="inlineStr">
+      <c r="G30" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -6156,7 +7395,7 @@
       <c r="F31" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="G31" s="9" t="inlineStr">
+      <c r="G31" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -6189,7 +7428,7 @@
       <c r="F32" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="G32" s="9" t="inlineStr">
+      <c r="G32" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -6222,7 +7461,7 @@
       <c r="F33" s="5" t="n">
         <v>37</v>
       </c>
-      <c r="G33" s="9" t="inlineStr">
+      <c r="G33" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -6288,7 +7527,7 @@
       <c r="F35" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="G35" s="9" t="inlineStr">
+      <c r="G35" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -6321,7 +7560,7 @@
       <c r="F36" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="G36" s="9" t="inlineStr">
+      <c r="G36" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -6354,7 +7593,7 @@
       <c r="F37" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="G37" s="9" t="inlineStr">
+      <c r="G37" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -6387,7 +7626,7 @@
       <c r="F38" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="G38" s="9" t="inlineStr">
+      <c r="G38" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -6453,7 +7692,7 @@
       <c r="F40" s="5" t="n">
         <v>48</v>
       </c>
-      <c r="G40" s="9" t="inlineStr">
+      <c r="G40" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -6486,7 +7725,7 @@
       <c r="F41" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G41" s="9" t="inlineStr">
+      <c r="G41" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -6519,7 +7758,7 @@
       <c r="F42" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G42" s="9" t="inlineStr">
+      <c r="G42" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -6849,7 +8088,7 @@
       <c r="F52" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="G52" s="9" t="inlineStr">
+      <c r="G52" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -6882,7 +8121,7 @@
       <c r="F53" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G53" s="9" t="inlineStr">
+      <c r="G53" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7146,7 +8385,7 @@
       <c r="F61" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G61" s="9" t="inlineStr">
+      <c r="G61" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7245,7 +8484,7 @@
       <c r="F64" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="G64" s="9" t="inlineStr">
+      <c r="G64" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7278,7 +8517,7 @@
       <c r="F65" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="G65" s="9" t="inlineStr">
+      <c r="G65" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7377,7 +8616,7 @@
       <c r="F68" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="G68" s="9" t="inlineStr">
+      <c r="G68" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7410,7 +8649,7 @@
       <c r="F69" s="5" t="n">
         <v>48</v>
       </c>
-      <c r="G69" s="9" t="inlineStr">
+      <c r="G69" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7443,7 +8682,7 @@
       <c r="F70" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G70" s="9" t="inlineStr">
+      <c r="G70" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7509,7 +8748,7 @@
       <c r="F72" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="G72" s="9" t="inlineStr">
+      <c r="G72" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7575,7 +8814,7 @@
       <c r="F74" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="G74" s="9" t="inlineStr">
+      <c r="G74" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7608,7 +8847,7 @@
       <c r="F75" s="5" t="n">
         <v>48</v>
       </c>
-      <c r="G75" s="9" t="inlineStr">
+      <c r="G75" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7674,7 +8913,7 @@
       <c r="F77" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="G77" s="9" t="inlineStr">
+      <c r="G77" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7740,7 +8979,7 @@
       <c r="F79" s="5" t="n">
         <v>48</v>
       </c>
-      <c r="G79" s="9" t="inlineStr">
+      <c r="G79" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7872,7 +9111,7 @@
       <c r="F83" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="G83" s="9" t="inlineStr">
+      <c r="G83" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7905,7 +9144,7 @@
       <c r="F84" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="G84" s="9" t="inlineStr">
+      <c r="G84" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7938,7 +9177,7 @@
       <c r="F85" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="G85" s="9" t="inlineStr">
+      <c r="G85" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -8004,7 +9243,7 @@
       <c r="F87" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G87" s="9" t="inlineStr">
+      <c r="G87" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -8136,7 +9375,7 @@
       <c r="F91" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="G91" s="9" t="inlineStr">
+      <c r="G91" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -8169,7 +9408,7 @@
       <c r="F92" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="G92" s="9" t="inlineStr">
+      <c r="G92" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -8301,7 +9540,7 @@
       <c r="F96" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G96" s="9" t="inlineStr">
+      <c r="G96" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -8730,7 +9969,7 @@
       <c r="F109" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="G109" s="9" t="inlineStr">
+      <c r="G109" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -8829,7 +10068,7 @@
       <c r="F112" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="G112" s="9" t="inlineStr">
+      <c r="G112" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -8961,7 +10200,7 @@
       <c r="F116" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G116" s="9" t="inlineStr">
+      <c r="G116" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -8994,7 +10233,7 @@
       <c r="F117" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="G117" s="9" t="inlineStr">
+      <c r="G117" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -9126,7 +10365,7 @@
       <c r="F121" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="G121" s="9" t="inlineStr">
+      <c r="G121" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -9357,7 +10596,7 @@
       <c r="F128" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="G128" s="9" t="inlineStr">
+      <c r="G128" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -9588,7 +10827,7 @@
       <c r="F135" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G135" s="9" t="inlineStr">
+      <c r="G135" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -14703,7 +15942,7 @@
       <c r="F290" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="G290" s="9" t="inlineStr">
+      <c r="G290" s="10" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -15737,7 +16976,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15992,13 +17231,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -16006,172 +17245,184 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>7 Day Kitchens, Keyword Research Workbook</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr"/>
+      <c r="B1" s="16" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>Prepared by</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="16" t="inlineStr">
         <is>
           <t>EmberTribe · SEO &amp; AI Growth Roadmap</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr"/>
-      <c r="B3" s="11" t="inlineStr"/>
+      <c r="A3" s="17" t="inlineStr"/>
+      <c r="B3" s="16" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>What's in here</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr"/>
+      <c r="B4" s="16" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Article Plan</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>The 120 articles in your 90-day plan: title, primary keyword, pillar, funnel stage, monthly demand, and difficulty (KD). 40 per month.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Service Pages</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>The recommended service-page architecture beyond Kitchen Remodeling + Kitchen Design: core kitchen, Kitchen + X combos (bath, walk-in pantry, scullery, laundry), segment pages (small/luxury/galley/open-concept), component pages (cabinets, refacing, countertops, islands), and suburb service-area pages. Prioritized P1/P2/P3. The blog articles link into these pages. Head-term volume is US topic demand; the local page captures the Charlotte + suburb + long-tail slice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Keyword Universe</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>The wider opportunity (top 320 on-strategy keywords). 'Yes (planned)' = covered by an article; 'Overflow' = held for later months.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Excluded</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>Keywords we deliberately left out, and why. Mostly competitor brands, wrong-city terms, and DIY/retail intent.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr"/>
-      <c r="B8" s="11" t="inlineStr"/>
-    </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr"/>
+      <c r="B9" s="16" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>A note on demand</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>Demand/mo blends two verified sources: SEMrush search volume for the local commercial terms, and your own Google Search Console monthly impressions for everything you already appear for. Both are real, not estimates.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr"/>
-      <c r="B10" s="11" t="inlineStr"/>
-    </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr"/>
+      <c r="B11" s="16" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>How to read the colors</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Pillar</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>Gold = Cost &amp; Budget · Blue = Design &amp; Materials · Green = Process &amp; Planning · Tan = Charlotte &amp; Local.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>KD (difficulty)</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>Green = easy (under 30) · Yellow = moderate (30-49) · Red = hard (50+). Lower is faster to rank.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Funnel</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>BoFu = decision-stage (ready to remodel) · MoFu = comparison · ToFu = inspiration / education.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="12" t="inlineStr"/>
-      <c r="B15" s="11" t="inlineStr"/>
-    </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr"/>
+      <c r="B16" s="16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>Why these pillars</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="B17" s="16" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Strategy</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B18" s="16" t="inlineStr">
         <is>
           <t>Win the local Charlotte and suburb searches first (your money pages), answer the cost and budget questions where your fixed-price model is the edge, build trust with process and timeline content, and cast a wide net with design and materials inspiration, all routed toward a quote through internal links.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr"/>
-      <c r="B18" s="11" t="inlineStr"/>
-    </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr"/>
+      <c r="B19" s="16" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Next step</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B20" s="16" t="inlineStr">
         <is>
           <t>Review the plan, then let's lock Month 1 and start production. Questions? Reply to the email this was shared from.</t>
         </is>

</xml_diff>

<commit_message>
7 Day Kitchens: rebuild content plan from Strategy Builder universe + refine service pages
Content plan now sourced from SEMrush Keyword Strategy Builder (real vol/KD):
kitchens-focus, net-new vs existing, topic caps (no cannibalization), stronger
semantic dedup, editorial titles, "US topic demand" labeled honestly.
Service pages: split Countertops -> Quartz (KD28) + Granite (KD36) easy wins,
retarget Backsplash. Deck slide 15 + Service Pages tab updated.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/7-day-kitchens/keyword-research.xlsx
+++ b/decks/7-day-kitchens/keyword-research.xlsx
@@ -90,17 +90,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00D9EAE2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00162f41"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F8D7DA"/>
       </patternFill>
     </fill>
     <fill>
@@ -123,7 +123,7 @@
   </cellStyleXfs>
   <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -138,14 +138,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -817,12 +817,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Kitchen Renovation Services Charlotte: Local Crews, Lifetime Warranty</t>
+          <t>Kitchen Remodeling Companies Charlotte: Local Crews, Lifetime Warranty</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>kitchen renovation services charlotte</t>
+          <t>kitchen remodeling companies charlotte</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -841,10 +841,10 @@
         </is>
       </c>
       <c r="G8" s="3" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -855,12 +855,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling South West Charlotte: One Local Crew, Start to Finish</t>
+          <t>Kitchen and Bath Remodeling in Charlotte, NC: One Crew, One Timeline</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>kitchen remodeling south west charlotte</t>
+          <t>kitchen and bath remodeling charlotte nc</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -882,7 +882,7 @@
         <v>40</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>7</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
@@ -1007,12 +1007,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>The Average Cost of a Kitchen Remodel, and Why Yours May Differ</t>
+          <t>Quartz Countertop Pricing: What Sets the Range</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>average cost of kitchen remodel</t>
+          <t>quartz price</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -1031,10 +1031,10 @@
         </is>
       </c>
       <c r="G13" s="3" t="n">
-        <v>10</v>
+        <v>880</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -1045,12 +1045,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Average Cost of a Full Kitchen Remodel: The Real Numbers for 2026</t>
+          <t>The Average Cost of a Kitchen Remodel, and Why Yours May Differ</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>average cost of a full kitchen remodel</t>
+          <t>average cost of kitchen remodel</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -1083,12 +1083,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Average Cost of Galley Kitchen Remodel: What to Know Before You Commit</t>
+          <t>How to Set a Kitchen Remodel Budget You Won't Blow Through</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>average cost of galley kitchen remodel</t>
+          <t>kitchen remodel budget</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1107,10 +1107,10 @@
         </is>
       </c>
       <c r="G15" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H15" s="4" t="n">
-        <v>24</v>
+        <v>1600</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="16">
@@ -1121,12 +1121,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Is Average Cost to Update a Kitchen Worth It?</t>
+          <t>What a Kitchen Island Costs to Build In</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>average cost to update a kitchen</t>
+          <t>kitchen island cost</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -1141,14 +1141,14 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G16" s="3" t="n">
-        <v>10</v>
+        <v>880</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17">
@@ -1159,12 +1159,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>How to Read a Kitchen Remodel Estimate, Line by Line</t>
+          <t>Budget Backsplash Ideas That Still Look High-End</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>kitchen estimate</t>
+          <t>cheap backsplash</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -1183,10 +1183,10 @@
         </is>
       </c>
       <c r="G17" s="3" t="n">
-        <v>61</v>
-      </c>
-      <c r="H17" s="6" t="n">
-        <v>48</v>
+        <v>480</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="18">
@@ -1197,12 +1197,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Getting a Kitchen Remodel Estimate: What to Expect</t>
+          <t>Budget-Friendly Kitchen Remodels: Smart Places to Save</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>kitchen remodel estimate</t>
+          <t>budget friendly kitchen remodel</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -1217,14 +1217,14 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G18" s="3" t="n">
-        <v>37</v>
+        <v>320</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19">
@@ -1235,12 +1235,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Kitchen Remodel Prices in 2026: What Sets the Range</t>
+          <t>Choosing Backsplash Prices Without Regret</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>kitchen prices</t>
+          <t>backsplash prices</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -1259,10 +1259,10 @@
         </is>
       </c>
       <c r="G19" s="3" t="n">
-        <v>24</v>
+        <v>140</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>48</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20">
@@ -1273,12 +1273,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>What a Kitchen Installation Estimate Should Include</t>
+          <t>Financing a Kitchen Remodel: Options Weighed Honestly</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>kitchen installation cost estimate</t>
+          <t>kitchen remodel financing</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -1297,7 +1297,7 @@
         </is>
       </c>
       <c r="G20" s="3" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="H20" s="6" t="n">
         <v>30</v>
@@ -1311,22 +1311,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>How to Set a Kitchen Remodel Budget You Won't Blow Through</t>
+          <t>Peel-and-Stick Backsplash: Quick Fix or False Economy?</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>kitchen remodel budget</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Cost &amp; Budget</t>
+          <t>peel and stick backsplash</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1335,10 +1335,10 @@
         </is>
       </c>
       <c r="G21" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H21" s="6" t="n">
-        <v>38</v>
+        <v>33100</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="22">
@@ -1349,12 +1349,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Kitchen and Laundry Room Combos: Designing the Two as One Project</t>
+          <t>Should Your Kitchen Have an Island? A Layout Guide</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>kitchen and laundry room remodel</t>
+          <t>kitchen island</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1373,10 +1373,10 @@
         </is>
       </c>
       <c r="G22" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H22" s="4" t="n">
-        <v>24</v>
+        <v>90500</v>
+      </c>
+      <c r="H22" s="8" t="n">
+        <v>52</v>
       </c>
     </row>
     <row r="23">
@@ -1387,12 +1387,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Kitchen Renovation, Start to Finish: A Homeowner's Overview</t>
+          <t>Kitchen Backsplash Ideas That Pull a Remodel Together</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>kitchen renovation</t>
+          <t>kitchen backsplash ideas</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -1402,19 +1402,19 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G23" s="3" t="n">
-        <v>232</v>
-      </c>
-      <c r="H23" s="6" t="n">
-        <v>48</v>
+        <v>18100</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="24">
@@ -1425,12 +1425,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Kitchen Design Ideas: Layouts, Light, and Lasting Style</t>
+          <t>Kitchen Island Ideas: Sizing, Seating, and Smart Storage</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>kitchen design ideas</t>
+          <t>kitchen island ideas</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -1449,10 +1449,10 @@
         </is>
       </c>
       <c r="G24" s="3" t="n">
+        <v>12100</v>
+      </c>
+      <c r="H24" s="6" t="n">
         <v>40</v>
-      </c>
-      <c r="H24" s="6" t="n">
-        <v>38</v>
       </c>
     </row>
     <row r="25">
@@ -1463,12 +1463,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Kitchen Backsplash Ideas That Pull a Remodel Together</t>
+          <t>Galley Kitchen Ideas: Big Function in a Narrow Footprint</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>kitchen backsplash ideas</t>
+          <t>galley kitchen ideas</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -1487,10 +1487,10 @@
         </is>
       </c>
       <c r="G25" s="3" t="n">
-        <v>40</v>
+        <v>3600</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="26">
@@ -1501,12 +1501,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Kitchen Flooring Options Ranked for Durability and Looks</t>
+          <t>Open-Concept Kitchens: When Knocking Down a Wall Pays Off</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>kitchen flooring options</t>
+          <t>open concept kitchen</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1525,10 +1525,10 @@
         </is>
       </c>
       <c r="G26" s="3" t="n">
-        <v>40</v>
+        <v>2400</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27">
@@ -1539,12 +1539,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Farmhouse Kitchen Ideas That Still Feel Fresh in 2026</t>
+          <t>Kitchen Layout Basics: Work Triangles, Walkways, and Flow</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>farmhouse kitchen ideas</t>
+          <t>kitchen layout</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
@@ -1559,14 +1559,14 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G27" s="3" t="n">
         <v>40</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28">
@@ -1577,12 +1577,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Choosing a Kitchen Faucet: Finishes, Features, and Value</t>
+          <t>Kitchen Lighting Ideas: Layering Task, Ambient, and Accent</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>kitchen faucet ideas</t>
+          <t>kitchen lighting ideas</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1615,12 +1615,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Small Kitchen Ideas: Making a Compact Space Feel Open</t>
+          <t>Modern Kitchen Design: Clean Lines Without the Cold Feel</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>small kitchen ideas</t>
+          <t>modern kitchen design</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G29" s="3" t="n">
@@ -1653,12 +1653,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Two-Tone Kitchen Cabinets: How to Mix Without a Mess</t>
+          <t>Pantry Ideas: Designing Storage That Earns Its Footprint</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>two tone kitchen cabinets</t>
+          <t>pantry ideas</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
@@ -1673,14 +1673,14 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G30" s="3" t="n">
         <v>40</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>30</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31">
@@ -1691,12 +1691,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Kitchen Storage Ideas That Use Every Inch</t>
+          <t>Two-Tone Kitchen Cabinets: How to Mix Without a Mess</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>kitchen storage ideas</t>
+          <t>two tone kitchen cabinets</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
@@ -1711,14 +1711,14 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G31" s="3" t="n">
         <v>40</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
     </row>
     <row r="32">
@@ -1767,22 +1767,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Waterfall Islands: The Statement Feature Worth the Splurge</t>
+          <t>Kitchen Remodel Contractors in Rock Hill, SC</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>waterfall island</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>Design &amp; Materials</t>
+          <t>contractor for kitchen remodel rock hill sc</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>Process &amp; Planning</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1791,10 +1791,10 @@
         </is>
       </c>
       <c r="G33" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H33" s="6" t="n">
-        <v>48</v>
+        <v>10</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="34">
@@ -1805,22 +1805,22 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Kitchen Countertops Compared: Quartz, Granite, and the Alternatives</t>
+          <t>Kitchen Renovation Contractors: What to Expect, Day by Day</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>kitchen countertops</t>
-        </is>
-      </c>
-      <c r="D34" s="7" t="inlineStr">
-        <is>
-          <t>Design &amp; Materials</t>
+          <t>kitchen renovation contractors</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>Process &amp; Planning</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1829,10 +1829,10 @@
         </is>
       </c>
       <c r="G34" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H34" s="6" t="n">
-        <v>48</v>
+        <v>2900</v>
+      </c>
+      <c r="H34" s="8" t="n">
+        <v>52</v>
       </c>
     </row>
     <row r="35">
@@ -1843,15 +1843,15 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Kitchen Remodel Contractors in Rock Hill, SC</t>
+          <t>Bathroom and Kitchen Contractors: What Separates Great From Cheap</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>contractor for kitchen remodel rock hill sc</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
+          <t>bathroom and kitchen contractors</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -1867,10 +1867,10 @@
         </is>
       </c>
       <c r="G35" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H35" s="4" t="n">
-        <v>24</v>
+        <v>390</v>
+      </c>
+      <c r="H35" s="6" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="36">
@@ -1881,34 +1881,34 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Kitchen Remodeler Gastonia: What Separates Great From Cheap</t>
+          <t>DIY Kitchen Furniture: The Process, Demystified</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>kitchen remodeler gastonia</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
+          <t>diy kitchen furniture</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G36" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H36" s="6" t="n">
-        <v>38</v>
+        <v>390</v>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="37">
@@ -1919,34 +1919,34 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Kitchen and Bath Remodeling Contractors: What Separates Great From Cheap</t>
+          <t>Tiny Kitchen Plans: Timelines, Trade-offs, and Questions to Ask</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>kitchen and bath remodeling contractors</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
+          <t>tiny kitchen plans</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G37" s="3" t="n">
-        <v>10</v>
+        <v>320</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38">
@@ -1957,34 +1957,34 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>How to Compare the Best Kitchen Remodel Contractors</t>
+          <t>Small Kitchen Plans: What Every Remodel Should Know</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>best kitchen remodel contractors</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
+          <t>small kitchen plans</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G38" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H38" s="6" t="n">
-        <v>30</v>
+        <v>170</v>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="39">
@@ -1995,34 +1995,34 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Kitchen Remodeler Eastway Park, Done the Fixed-Price Way</t>
+          <t>Open Kitchen Living Room: Timelines, Trade-offs, and Questions to Ask</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>kitchen remodeler eastway park</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
+          <t>open kitchen living room</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G39" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H39" s="6" t="n">
-        <v>30</v>
+        <v>720</v>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="40">
@@ -2033,31 +2033,31 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Kitchen Remodeler Contractor: What to Expect, Day by Day</t>
+          <t>The Kitchen Remodel Checklist Every Homeowner Should Use</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>kitchen remodeler contractor</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
+          <t>kitchen remodel checklist</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G40" s="3" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="H40" s="6" t="n">
         <v>38</v>
@@ -2071,31 +2071,31 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>The Kitchen Remodel Checklist Every Homeowner Should Use</t>
+          <t>Kitchen Remodeling Timeline: What It Takes, Start to Finish</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>kitchen remodel checklist</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
+          <t>kitchen remodeling timeline</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G41" s="3" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="H41" s="6" t="n">
         <v>38</v>
@@ -2109,7 +2109,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Kitchen Design and Build Charlotte NC: What the Process Looks Like Here</t>
+          <t>Kitchen Design and Build Charlotte NC: A Faster Path to Your Dream Kitchen</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2337,12 +2337,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Ballantyne Kitchen Remodeling: Premium Results Without the Wait</t>
+          <t>Kitchen Renovation Services Charlotte: What the Process Looks Like Here</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>kitchen remodeling ballantyne</t>
+          <t>kitchen renovation services charlotte</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2361,10 +2361,10 @@
         </is>
       </c>
       <c r="G48" s="3" t="n">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="H48" s="4" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="49">
@@ -2375,12 +2375,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Kitchen Remodelers Charlotte NC: A Faster Path to Your Dream Kitchen</t>
+          <t>Kitchen Remodeling South West Charlotte: One Local Crew, Start to Finish</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>kitchen remodelers charlotte nc</t>
+          <t>kitchen remodeling south west charlotte</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -2399,10 +2399,10 @@
         </is>
       </c>
       <c r="G49" s="3" t="n">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="H49" s="4" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
     </row>
     <row r="50">
@@ -2489,12 +2489,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Approximate Cost of Kitchen Remodel: Budget, Mid-Range, and High-End Compared</t>
+          <t>What Quartz Countertops Cost, Installed</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>approximate cost of kitchen remodel</t>
+          <t>cost of quartz countertops</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
@@ -2513,10 +2513,10 @@
         </is>
       </c>
       <c r="G52" s="3" t="n">
-        <v>10</v>
+        <v>2900</v>
       </c>
       <c r="H52" s="4" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="53">
@@ -2527,12 +2527,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Average Cost of a Kitchen Remodel 2024: What Drives the Final Price</t>
+          <t>Small Kitchen Remodels: Where the Budget Goes</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>average cost of a kitchen remodel 2024</t>
+          <t>small kitchen remodel price</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
@@ -2547,14 +2547,14 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G53" s="3" t="n">
-        <v>10</v>
+        <v>480</v>
       </c>
       <c r="H53" s="4" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="54">
@@ -2565,12 +2565,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Average Cost of Large Kitchen Remodel: Where Most Homeowners Get It Wrong</t>
+          <t>How Much Space to Leave Between Counter and Island</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>average cost of large kitchen remodel</t>
+          <t>how much space between counter and island</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
@@ -2585,14 +2585,14 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G54" s="3" t="n">
-        <v>10</v>
+        <v>320</v>
       </c>
       <c r="H54" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="55">
@@ -2603,12 +2603,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling Cost: Where the Money Goes, and Where to Save</t>
+          <t>Cheap Backsplash Options: What to Know Before You Commit</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>kitchen remodeling cost</t>
+          <t>cheap backsplash options</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
@@ -2623,14 +2623,14 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G55" s="3" t="n">
-        <v>60</v>
-      </c>
-      <c r="H55" s="6" t="n">
-        <v>38</v>
+        <v>260</v>
+      </c>
+      <c r="H55" s="4" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="56">
@@ -2641,12 +2641,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Comparing Kitchen Remodel Quotes: A Side-by-Side Guide</t>
+          <t>Laminate Countertops: The Budget-Friendly Counter Option</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>compare kitchen prices</t>
+          <t>laminate countertop cost</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
@@ -2665,10 +2665,10 @@
         </is>
       </c>
       <c r="G56" s="3" t="n">
-        <v>15</v>
+        <v>880</v>
       </c>
       <c r="H56" s="6" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="57">
@@ -2679,12 +2679,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Financing a Kitchen Remodel: Options Weighed Honestly</t>
+          <t>A Kitchen Makeover on a Budget: What's Realistic</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>kitchen remodel financing</t>
+          <t>kitchen makeover on a budget</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
@@ -2699,14 +2699,14 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G57" s="3" t="n">
-        <v>10</v>
+        <v>390</v>
       </c>
       <c r="H57" s="6" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="58">
@@ -2717,22 +2717,22 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>What Full-Service Kitchen Remodeling Actually Covers</t>
+          <t>Small Kitchen Remodels on a Budget: What to Budget Before You Start</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>kitchen remodeling services</t>
-        </is>
-      </c>
-      <c r="D58" s="7" t="inlineStr">
-        <is>
-          <t>Design &amp; Materials</t>
+          <t>small kitchen remodels on a budget</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Cost &amp; Budget</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2741,10 +2741,10 @@
         </is>
       </c>
       <c r="G58" s="3" t="n">
-        <v>38</v>
-      </c>
-      <c r="H58" s="6" t="n">
-        <v>38</v>
+        <v>260</v>
+      </c>
+      <c r="H58" s="4" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="59">
@@ -2755,17 +2755,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Choosing Kitchen Cabinets: Styles, Finishes, and What Lasts</t>
+          <t>Kitchen Renovation Cost: A Room-by-Room Money Map</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>kitchen cabinets</t>
-        </is>
-      </c>
-      <c r="D59" s="7" t="inlineStr">
-        <is>
-          <t>Design &amp; Materials</t>
+          <t>kitchen renovation cost</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Cost &amp; Budget</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2782,7 +2782,7 @@
         <v>10</v>
       </c>
       <c r="H59" s="6" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
     </row>
     <row r="60">
@@ -2793,12 +2793,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Kitchen Cabinet Installation: How It's Done Right</t>
+          <t>Cabinet Refacing in Charlotte, NC: When It Makes Sense</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>kitchen cabinet installation</t>
+          <t>cabinet refacing charlotte nc</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2817,10 +2817,10 @@
         </is>
       </c>
       <c r="G60" s="3" t="n">
-        <v>96</v>
-      </c>
-      <c r="H60" s="6" t="n">
-        <v>38</v>
+        <v>102</v>
+      </c>
+      <c r="H60" s="4" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="61">
@@ -2831,12 +2831,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Quartz vs Granite Countertops: Which Wins for Your Kitchen</t>
+          <t>Kitchen and Laundry Room Combos: Designing the Two as One Project</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>quartz vs granite</t>
+          <t>kitchen and laundry room remodel</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
@@ -2846,7 +2846,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2857,8 +2857,8 @@
       <c r="G61" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="H61" s="6" t="n">
-        <v>38</v>
+      <c r="H61" s="4" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="62">
@@ -2869,12 +2869,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Kitchen Layout Basics: Work Triangles, Walkways, and Flow</t>
+          <t>Butcher Block Countertops: Warm Looks, Real Trade-offs</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>kitchen layout</t>
+          <t>butcher block countertops</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2893,10 +2893,10 @@
         </is>
       </c>
       <c r="G62" s="3" t="n">
-        <v>40</v>
+        <v>40500</v>
       </c>
       <c r="H62" s="6" t="n">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="63">
@@ -2907,12 +2907,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Kitchen Lighting Ideas: Layering Task, Ambient, and Accent</t>
+          <t>Adding a Scullery to Your Kitchen: The Hidden Prep-Space Trend</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>kitchen lighting ideas</t>
+          <t>kitchen scullery</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
@@ -2927,14 +2927,14 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G63" s="3" t="n">
-        <v>40</v>
+        <v>18100</v>
       </c>
       <c r="H63" s="6" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="64">
@@ -2945,12 +2945,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Modern Kitchen Design: Clean Lines Without the Cold Feel</t>
+          <t>Subway Tile Backsplash: The Timeless Default, Done Right</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>modern kitchen design</t>
+          <t>subway tile backsplash</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -2969,10 +2969,10 @@
         </is>
       </c>
       <c r="G64" s="3" t="n">
-        <v>40</v>
+        <v>12100</v>
       </c>
       <c r="H64" s="6" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
     </row>
     <row r="65">
@@ -2983,12 +2983,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Pantry Ideas: Designing Storage That Earns Its Footprint</t>
+          <t>Kitchen Storage Ideas That Use Every Inch</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>pantry ideas</t>
+          <t>kitchen storage ideas</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
@@ -3007,10 +3007,10 @@
         </is>
       </c>
       <c r="G65" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H65" s="6" t="n">
-        <v>48</v>
+        <v>2900</v>
+      </c>
+      <c r="H65" s="8" t="n">
+        <v>52</v>
       </c>
     </row>
     <row r="66">
@@ -3021,12 +3021,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Kitchen Paint Colors That Flatter Cabinets and Counters</t>
+          <t>Kitchen Cabinet Styles: Shaker, Flat-Panel, and Beyond</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>kitchen paint colors</t>
+          <t>kitchen cabinet styles</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
@@ -3045,10 +3045,10 @@
         </is>
       </c>
       <c r="G66" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H66" s="6" t="n">
-        <v>38</v>
+        <v>2400</v>
+      </c>
+      <c r="H66" s="4" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="67">
@@ -3059,12 +3059,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Kitchen Appliances: Where to Splurge and Where to Save</t>
+          <t>Kitchen Design Ideas: Layouts, Light, and Lasting Style</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>kitchen appliances</t>
+          <t>kitchen design ideas</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
@@ -3074,19 +3074,19 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G67" s="3" t="n">
         <v>40</v>
       </c>
       <c r="H67" s="6" t="n">
-        <v>48</v>
+        <v>38</v>
       </c>
     </row>
     <row r="68">
@@ -3097,12 +3097,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Adding a Scullery to Your Kitchen: The Hidden Prep-Space Trend</t>
+          <t>Kitchen Cabinet Colors: What's Timeless vs What's Trendy</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>kitchen scullery</t>
+          <t>kitchen cabinet colors</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
@@ -3124,7 +3124,7 @@
         <v>40</v>
       </c>
       <c r="H68" s="6" t="n">
-        <v>48</v>
+        <v>38</v>
       </c>
     </row>
     <row r="69">
@@ -3135,12 +3135,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Kitchen and Mudroom Combos: A Smarter Family Entryway</t>
+          <t>Kitchen Trends 2026: Bold Cabinets, Brass, and What to Skip</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>kitchen and mudroom</t>
+          <t>kitchen trends 2026</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
@@ -3155,7 +3155,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G69" s="3" t="n">
@@ -3173,12 +3173,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Galley Kitchen Ideas: Big Function in a Narrow Footprint</t>
+          <t>Kitchen Sink Ideas: Materials, Mounts, and the Right Size</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>galley kitchen ideas</t>
+          <t>kitchen sink ideas</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
@@ -3211,12 +3211,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>White Kitchen Cabinets: Why They Endure, and How to Keep Them Clean</t>
+          <t>Kitchen Paint Colors That Flatter Cabinets and Counters</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>white kitchen cabinets</t>
+          <t>kitchen paint colors</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
@@ -3235,7 +3235,7 @@
         </is>
       </c>
       <c r="G71" s="3" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="H71" s="6" t="n">
         <v>38</v>
@@ -3249,22 +3249,22 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Kitchen Remodeler Rock Hill: Done Right the First Time</t>
+          <t>Kitchen Appliances: Where to Splurge and Where to Save</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>kitchen remodeler rock hill</t>
-        </is>
-      </c>
-      <c r="D72" s="8" t="inlineStr">
-        <is>
-          <t>Process &amp; Planning</t>
+          <t>kitchen appliances</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3273,10 +3273,10 @@
         </is>
       </c>
       <c r="G72" s="3" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="H72" s="6" t="n">
-        <v>30</v>
+        <v>48</v>
       </c>
     </row>
     <row r="73">
@@ -3287,22 +3287,22 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Kitchen Remodeler Concord, Done the Fixed-Price Way</t>
+          <t>Kitchen and Mudroom Combos: A Smarter Family Entryway</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>kitchen remodeler concord</t>
-        </is>
-      </c>
-      <c r="D73" s="8" t="inlineStr">
-        <is>
-          <t>Process &amp; Planning</t>
+          <t>kitchen and mudroom</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3311,7 +3311,7 @@
         </is>
       </c>
       <c r="G73" s="3" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="H73" s="6" t="n">
         <v>38</v>
@@ -3325,15 +3325,15 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Finding Local Contractors for a Kitchen Remodel</t>
+          <t>Kitchen Contractors: Done Right the First Time</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>local contractors for kitchen remodel</t>
-        </is>
-      </c>
-      <c r="D74" s="8" t="inlineStr">
+          <t>kitchen contractors</t>
+        </is>
+      </c>
+      <c r="D74" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -3349,10 +3349,10 @@
         </is>
       </c>
       <c r="G74" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H74" s="4" t="n">
-        <v>24</v>
+        <v>2400</v>
+      </c>
+      <c r="H74" s="8" t="n">
+        <v>53</v>
       </c>
     </row>
     <row r="75">
@@ -3363,15 +3363,15 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Choosing a Contractor for Your Kitchen Renovation</t>
+          <t>Local Kitchen Remodelers: The Questions to Ask First</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>contractor for kitchen renovation</t>
-        </is>
-      </c>
-      <c r="D75" s="8" t="inlineStr">
+          <t>local kitchen remodelers</t>
+        </is>
+      </c>
+      <c r="D75" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -3387,10 +3387,10 @@
         </is>
       </c>
       <c r="G75" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H75" s="6" t="n">
-        <v>30</v>
+        <v>320</v>
+      </c>
+      <c r="H75" s="8" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="76">
@@ -3401,15 +3401,15 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Best Kitchen Remodeler: The Questions to Ask First</t>
+          <t>How to Compare the Best Kitchen Remodel Contractors</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>best kitchen remodeler</t>
-        </is>
-      </c>
-      <c r="D76" s="8" t="inlineStr">
+          <t>best kitchen remodel contractors</t>
+        </is>
+      </c>
+      <c r="D76" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -3428,7 +3428,7 @@
         <v>10</v>
       </c>
       <c r="H76" s="6" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
     </row>
     <row r="77">
@@ -3439,15 +3439,15 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>How to Plan a Kitchen Remodel Before Demo Day</t>
+          <t>How to Prepare Your Home for a Kitchen Remodel</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>how to plan a kitchen remodel</t>
-        </is>
-      </c>
-      <c r="D77" s="8" t="inlineStr">
+          <t>how to prepare for a kitchen remodel</t>
+        </is>
+      </c>
+      <c r="D77" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -3463,7 +3463,7 @@
         </is>
       </c>
       <c r="G77" s="3" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="H77" s="4" t="n">
         <v>24</v>
@@ -3477,15 +3477,15 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>How to Prepare Your Home for a Kitchen Remodel</t>
+          <t>DIY Kitchen Cupboards: A Homeowner's Walkthrough</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>how to prepare for a kitchen remodel</t>
-        </is>
-      </c>
-      <c r="D78" s="8" t="inlineStr">
+          <t>diy kitchen cupboards</t>
+        </is>
+      </c>
+      <c r="D78" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -3501,10 +3501,10 @@
         </is>
       </c>
       <c r="G78" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H78" s="4" t="n">
-        <v>24</v>
+        <v>880</v>
+      </c>
+      <c r="H78" s="6" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="79">
@@ -3515,34 +3515,34 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Kitchen Demolition: What Tear-Out Day Actually Involves</t>
+          <t>Galley Kitchen Plans: How to Pick the Right Pro</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>kitchen demolition</t>
-        </is>
-      </c>
-      <c r="D79" s="8" t="inlineStr">
+          <t>galley kitchen plans</t>
+        </is>
+      </c>
+      <c r="D79" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G79" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H79" s="6" t="n">
-        <v>48</v>
+        <v>720</v>
+      </c>
+      <c r="H79" s="4" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="80">
@@ -3553,22 +3553,22 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling Timeline: Timelines, Trade-offs, and Questions to Ask</t>
+          <t>Kitchen Demolition: What Tear-Out Day Actually Involves</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>kitchen remodeling timeline</t>
-        </is>
-      </c>
-      <c r="D80" s="8" t="inlineStr">
+          <t>kitchen demolition</t>
+        </is>
+      </c>
+      <c r="D80" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3577,10 +3577,10 @@
         </is>
       </c>
       <c r="G80" s="3" t="n">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="H80" s="6" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="81">
@@ -3599,7 +3599,7 @@
           <t>order of kitchen remodel</t>
         </is>
       </c>
-      <c r="D81" s="8" t="inlineStr">
+      <c r="D81" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -3819,12 +3819,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling Companies Charlotte: Fixed Pricing, Finished in 7 Days</t>
+          <t>Kitchen Remodeling Services Charlotte: Fixed Pricing, Finished in 7 Days</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>kitchen remodeling companies charlotte</t>
+          <t>kitchen remodeling services charlotte</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -3843,10 +3843,10 @@
         </is>
       </c>
       <c r="G87" s="3" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H87" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="88">
@@ -3857,12 +3857,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Kitchen and Bath Remodeling in Charlotte, NC: One Crew, One Timeline</t>
+          <t>Ballantyne Kitchen Remodeling: Premium Results Without the Wait</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>kitchen and bath remodeling charlotte nc</t>
+          <t>kitchen remodeling ballantyne</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -3998,7 +3998,7 @@
         <v>10</v>
       </c>
       <c r="H91" s="4" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="92">
@@ -4009,12 +4009,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Average Cost of a Complete Kitchen Remodel: Where the Money Goes, and Where to Save</t>
+          <t>What Granite Countertops Cost, Installed</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>average cost of a complete kitchen remodel</t>
+          <t>cost of granite countertops</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
@@ -4029,14 +4029,14 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G92" s="3" t="n">
-        <v>10</v>
+        <v>2900</v>
       </c>
       <c r="H92" s="4" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="93">
@@ -4047,12 +4047,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Average Cost of a New Kitchen Remodel: The Numbers Behind the Choice</t>
+          <t>What a Small Kitchen Remodel Really Costs</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>average cost of a new kitchen remodel</t>
+          <t>average cost of small kitchen remodel</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
@@ -4067,11 +4067,11 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G93" s="3" t="n">
-        <v>10</v>
+        <v>390</v>
       </c>
       <c r="H93" s="4" t="n">
         <v>24</v>
@@ -4085,12 +4085,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Average Cost of Redoing a Kitchen: A 2026 Buyer's Guide</t>
+          <t>How Much for a Small Kitchen Renovation: What to Weigh First</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>average cost of redoing a kitchen</t>
+          <t>how much for a small kitchen renovation</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
@@ -4105,14 +4105,14 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G94" s="3" t="n">
-        <v>10</v>
+        <v>260</v>
       </c>
       <c r="H94" s="4" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="95">
@@ -4123,12 +4123,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Affordable Kitchen Remodels: Where to Save Without Regret</t>
+          <t>Inexpensive Kitchen Renovations: A Straight Comparison for Homeowners</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>affordable kitchen remodel</t>
+          <t>inexpensive kitchen renovations</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
@@ -4143,14 +4143,14 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G95" s="3" t="n">
-        <v>63</v>
+        <v>1900</v>
       </c>
       <c r="H95" s="6" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="96">
@@ -4161,12 +4161,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>What Drives Your Kitchen Remodel Price: A Cost-Factor Guide</t>
+          <t>Cheap Backsplash Ideas: A Plain-English Cost Primer</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>kitchen remodel price</t>
+          <t>cheap backsplash ideas</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -4185,10 +4185,10 @@
         </is>
       </c>
       <c r="G96" s="3" t="n">
-        <v>40</v>
+        <v>880</v>
       </c>
       <c r="H96" s="6" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
     </row>
     <row r="97">
@@ -4199,12 +4199,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>What a Free Kitchen Remodel Estimate Should Tell You</t>
+          <t>How Much Are Kitchen Cupboards: Budget, Mid-Range, and High-End</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>free kitchen remodel estimate</t>
+          <t>how much are kitchen cupboards</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
@@ -4219,14 +4219,14 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G97" s="3" t="n">
-        <v>30</v>
+        <v>720</v>
       </c>
       <c r="H97" s="6" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="98">
@@ -4237,12 +4237,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>What a Brand-New Kitchen Costs vs a Remodel</t>
+          <t>Cost of New Kitchen: What Sets the Final Number</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>new kitchen prices</t>
+          <t>cost of new kitchen</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
@@ -4257,14 +4257,14 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G98" s="3" t="n">
-        <v>15</v>
+        <v>390</v>
       </c>
       <c r="H98" s="6" t="n">
-        <v>38</v>
+        <v>47</v>
       </c>
     </row>
     <row r="99">
@@ -4275,17 +4275,17 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Kitchen Renovation Cost: A Room-by-Room Money Map</t>
+          <t>Choosing Kitchen Cabinets: Styles, Finishes, and What Lasts</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>kitchen renovation cost</t>
-        </is>
-      </c>
-      <c r="D99" s="5" t="inlineStr">
-        <is>
-          <t>Cost &amp; Budget</t>
+          <t>kitchen cabinets</t>
+        </is>
+      </c>
+      <c r="D99" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4299,10 +4299,10 @@
         </is>
       </c>
       <c r="G99" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H99" s="6" t="n">
-        <v>30</v>
+        <v>165000</v>
+      </c>
+      <c r="H99" s="8" t="n">
+        <v>55</v>
       </c>
     </row>
     <row r="100">
@@ -4313,12 +4313,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Cabinet Refacing in Charlotte, NC: When It Makes Sense</t>
+          <t>Quartz Countertops: Why They Dominate Modern Kitchens</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>cabinet refacing charlotte nc</t>
+          <t>quartz countertops</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
@@ -4328,7 +4328,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -4337,10 +4337,10 @@
         </is>
       </c>
       <c r="G100" s="3" t="n">
-        <v>102</v>
+        <v>90500</v>
       </c>
       <c r="H100" s="4" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="101">
@@ -4351,12 +4351,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Kitchen Remodel Before and After: What a Week Can Change</t>
+          <t>Kitchen Countertops Compared: Quartz, Granite, and the Alternatives</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>kitchen remodel before and after</t>
+          <t>kitchen countertops</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
@@ -4366,19 +4366,19 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G101" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H101" s="4" t="n">
-        <v>24</v>
+        <v>33100</v>
+      </c>
+      <c r="H101" s="6" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="102">
@@ -4389,12 +4389,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling 101: What the Project Really Involves</t>
+          <t>Small Kitchen Ideas: Making a Compact Space Feel Open</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>kitchen remodeling</t>
+          <t>small kitchen ideas</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
@@ -4404,19 +4404,19 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G102" s="3" t="n">
-        <v>374</v>
+        <v>14800</v>
       </c>
       <c r="H102" s="6" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="103">
@@ -4427,12 +4427,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Kitchen Island Ideas: Sizing, Seating, and Smart Storage</t>
+          <t>Kitchen Gadgets: What Designers Pick and Why</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>kitchen island ideas</t>
+          <t>kitchen gadgets</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
@@ -4442,19 +4442,19 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G103" s="3" t="n">
-        <v>40</v>
+        <v>9900</v>
       </c>
       <c r="H103" s="6" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="104">
@@ -4465,12 +4465,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Kitchen Cabinet Colors: What's Timeless vs What's Trendy</t>
+          <t>Waterfall Islands: The Statement Feature Worth the Splurge</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>kitchen cabinet colors</t>
+          <t>waterfall island</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
@@ -4489,10 +4489,10 @@
         </is>
       </c>
       <c r="G104" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H104" s="6" t="n">
-        <v>38</v>
+        <v>2900</v>
+      </c>
+      <c r="H104" s="4" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="105">
@@ -4503,12 +4503,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Kitchen Trends 2026: Bold Cabinets, Brass, and What to Skip</t>
+          <t>Kitchen Remodel Before and After: What a Week Can Change</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>kitchen trends 2026</t>
+          <t>kitchen remodel before and after</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
@@ -4527,10 +4527,10 @@
         </is>
       </c>
       <c r="G105" s="3" t="n">
-        <v>40</v>
+        <v>590</v>
       </c>
       <c r="H105" s="6" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
     </row>
     <row r="106">
@@ -4541,12 +4541,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Kitchen Sink Ideas: Materials, Mounts, and the Right Size</t>
+          <t>Quartz vs Granite Countertops: Which Wins for Your Kitchen</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>kitchen sink ideas</t>
+          <t>quartz vs granite</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
@@ -4556,12 +4556,12 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G106" s="3" t="n">
@@ -4579,12 +4579,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Open-Concept Kitchens: When Knocking Down a Wall Pays Off</t>
+          <t>Kitchen Flooring Options Ranked for Durability and Looks</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>open concept kitchen</t>
+          <t>kitchen flooring options</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
@@ -4594,7 +4594,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -4617,12 +4617,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Cabinet Hardware: The Small Detail That Sets the Tone</t>
+          <t>Farmhouse Kitchen Ideas That Still Feel Fresh in 2026</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>cabinet hardware ideas</t>
+          <t>farmhouse kitchen ideas</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
@@ -4655,12 +4655,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Butcher Block Countertops: Warm Looks, Real Trade-offs</t>
+          <t>Choosing a Kitchen Faucet: Finishes, Features, and Value</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>butcher block countertops</t>
+          <t>kitchen faucet ideas</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
@@ -4675,7 +4675,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G109" s="3" t="n">
@@ -4693,12 +4693,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Butler's Pantry Ideas: A Kitchen Upgrade That Adds Real Value</t>
+          <t>Cabinet Hardware: The Small Detail That Sets the Tone</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>butler pantry ideas</t>
+          <t>cabinet hardware ideas</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
@@ -4731,12 +4731,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Kitchen Cabinet Styles: Shaker, Flat-Panel, and Beyond</t>
+          <t>Butler's Pantry Ideas: A Kitchen Upgrade That Adds Real Value</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>kitchen cabinet styles</t>
+          <t>butler pantry ideas</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
@@ -4751,7 +4751,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G111" s="3" t="n">
@@ -4769,12 +4769,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Quartz Countertops: Why They Dominate Modern Kitchens</t>
+          <t>White Kitchen Cabinets: Why They Endure, and How to Keep Them Clean</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>quartz countertops</t>
+          <t>white kitchen cabinets</t>
         </is>
       </c>
       <c r="D112" s="7" t="inlineStr">
@@ -4784,7 +4784,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -4796,7 +4796,7 @@
         <v>10</v>
       </c>
       <c r="H112" s="6" t="n">
-        <v>48</v>
+        <v>38</v>
       </c>
     </row>
     <row r="113">
@@ -4807,15 +4807,15 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Kitchen Remodeler Davidson: A No-Nonsense Buyer's Guide</t>
+          <t>Finding Local Contractors for a Kitchen Remodel</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>kitchen remodeler davidson</t>
-        </is>
-      </c>
-      <c r="D113" s="8" t="inlineStr">
+          <t>local contractors for kitchen remodel</t>
+        </is>
+      </c>
+      <c r="D113" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -4833,8 +4833,8 @@
       <c r="G113" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="H113" s="6" t="n">
-        <v>38</v>
+      <c r="H113" s="4" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="114">
@@ -4845,15 +4845,15 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>What Separates a Great Kitchen Remodeler From the Rest</t>
+          <t>Kitchen Bath Contractor: A No-Nonsense Buyer's Guide</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>kitchen remodeler</t>
-        </is>
-      </c>
-      <c r="D114" s="8" t="inlineStr">
+          <t>kitchen bath contractor</t>
+        </is>
+      </c>
+      <c r="D114" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -4869,10 +4869,10 @@
         </is>
       </c>
       <c r="G114" s="3" t="n">
-        <v>151</v>
+        <v>480</v>
       </c>
       <c r="H114" s="6" t="n">
-        <v>48</v>
+        <v>39</v>
       </c>
     </row>
     <row r="115">
@@ -4883,15 +4883,15 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>What a Kitchen Contractor Handles on a Remodel</t>
+          <t>What Separates a Great Kitchen Remodeler From the Rest</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>kitchen contractor</t>
-        </is>
-      </c>
-      <c r="D115" s="8" t="inlineStr">
+          <t>kitchen remodeler</t>
+        </is>
+      </c>
+      <c r="D115" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -4907,7 +4907,7 @@
         </is>
       </c>
       <c r="G115" s="3" t="n">
-        <v>36</v>
+        <v>151</v>
       </c>
       <c r="H115" s="6" t="n">
         <v>48</v>
@@ -4921,34 +4921,34 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>A Homeowner's Guide to Kitchen Remodeler East Shoreham</t>
+          <t>Kitchen Cupboard Plans: What It Takes, Start to Finish</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>kitchen remodeler east shoreham</t>
-        </is>
-      </c>
-      <c r="D116" s="8" t="inlineStr">
+          <t>kitchen cupboard plans</t>
+        </is>
+      </c>
+      <c r="D116" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G116" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H116" s="6" t="n">
-        <v>30</v>
+        <v>320</v>
+      </c>
+      <c r="H116" s="4" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="117">
@@ -4959,34 +4959,34 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Kitchen Addition Contractors: What to Know Before You Commit</t>
+          <t>How to Plan a Kitchen Remodel Before Demo Day</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>kitchen addition contractors</t>
-        </is>
-      </c>
-      <c r="D117" s="8" t="inlineStr">
+          <t>how to plan a kitchen remodel</t>
+        </is>
+      </c>
+      <c r="D117" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G117" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H117" s="6" t="n">
-        <v>38</v>
+        <v>40</v>
+      </c>
+      <c r="H117" s="4" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="118">
@@ -4997,15 +4997,15 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Kitchen Remodel Order of Steps: Timelines, Trade-offs, and Questions to Ask</t>
+          <t>Open Kitchen Plans: How to Pick the Right Pro</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>kitchen remodel order of steps</t>
-        </is>
-      </c>
-      <c r="D118" s="8" t="inlineStr">
+          <t>open kitchen plans</t>
+        </is>
+      </c>
+      <c r="D118" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -5017,14 +5017,14 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G118" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="H118" s="4" t="n">
-        <v>24</v>
+        <v>260</v>
+      </c>
+      <c r="H118" s="6" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="119">
@@ -5043,7 +5043,7 @@
           <t>kitchen remodel permits</t>
         </is>
       </c>
-      <c r="D119" s="8" t="inlineStr">
+      <c r="D119" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -5081,7 +5081,7 @@
           <t>kitchen remodel contractor questions</t>
         </is>
       </c>
-      <c r="D120" s="8" t="inlineStr">
+      <c r="D120" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -5119,7 +5119,7 @@
           <t>kitchen renovation timeline</t>
         </is>
       </c>
-      <c r="D121" s="8" t="inlineStr">
+      <c r="D121" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -5152,7 +5152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5214,7 +5214,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -5245,7 +5245,7 @@
           <t>Buyer</t>
         </is>
       </c>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>Have — expand</t>
         </is>
@@ -5257,7 +5257,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -5280,7 +5280,7 @@
       <c r="E3" s="3" t="n">
         <v>22200</v>
       </c>
-      <c r="F3" s="11" t="n">
+      <c r="F3" s="8" t="n">
         <v>65</v>
       </c>
       <c r="G3" t="inlineStr">
@@ -5288,7 +5288,7 @@
           <t>Buyer</t>
         </is>
       </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>Have — expand</t>
         </is>
@@ -5300,7 +5300,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -5343,7 +5343,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -5386,7 +5386,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -5429,7 +5429,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -5472,7 +5472,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -5503,7 +5503,7 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="H8" s="11" t="inlineStr">
         <is>
           <t>Have</t>
         </is>
@@ -5515,7 +5515,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -5548,7 +5548,7 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="H9" s="10" t="inlineStr">
+      <c r="H9" s="11" t="inlineStr">
         <is>
           <t>Have</t>
         </is>
@@ -5560,7 +5560,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -5591,7 +5591,7 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="H10" s="10" t="inlineStr">
+      <c r="H10" s="11" t="inlineStr">
         <is>
           <t>Have — optimize</t>
         </is>
@@ -5626,7 +5626,7 @@
       <c r="E11" s="3" t="n">
         <v>9900</v>
       </c>
-      <c r="F11" s="11" t="n">
+      <c r="F11" s="8" t="n">
         <v>50</v>
       </c>
       <c r="G11" t="inlineStr">
@@ -5798,7 +5798,7 @@
       <c r="E15" s="3" t="n">
         <v>8100</v>
       </c>
-      <c r="F15" s="11" t="n">
+      <c r="F15" s="8" t="n">
         <v>54</v>
       </c>
       <c r="G15" t="inlineStr">
@@ -5894,7 +5894,7 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="H17" s="10" t="inlineStr">
+      <c r="H17" s="11" t="inlineStr">
         <is>
           <t>Have — optimize</t>
         </is>
@@ -5939,7 +5939,7 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="H18" s="10" t="inlineStr">
+      <c r="H18" s="11" t="inlineStr">
         <is>
           <t>Have — optimize</t>
         </is>
@@ -6064,7 +6064,7 @@
       <c r="E21" s="3" t="n">
         <v>1600</v>
       </c>
-      <c r="F21" s="11" t="n">
+      <c r="F21" s="8" t="n">
         <v>58</v>
       </c>
       <c r="G21" t="inlineStr">
@@ -6084,9 +6084,9 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -6096,19 +6096,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Kitchen Countertops</t>
+          <t>Quartz Countertops</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>kitchen countertops</t>
+          <t>quartz countertops</t>
         </is>
       </c>
       <c r="E22" s="3" t="n">
-        <v>40500</v>
-      </c>
-      <c r="F22" s="11" t="n">
-        <v>58</v>
+        <v>90500</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>28</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -6122,14 +6122,14 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Massive demand; feature-as-service that funnels to full remodels.</t>
+          <t>EASY WIN (KD 28) on the #1 countertop material. The real countertop money page.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -6139,19 +6139,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Kitchen Islands</t>
+          <t>Granite Countertops</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>kitchen island</t>
+          <t>granite countertops</t>
         </is>
       </c>
       <c r="E23" s="3" t="n">
-        <v>90500</v>
-      </c>
-      <c r="F23" s="11" t="n">
-        <v>61</v>
+        <v>60500</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>36</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -6165,7 +6165,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Highest demand of all (90.5K); high KD. Feature page funneling to remodels.</t>
+          <t>Winnable (KD 36). Pair with quartz under a Countertops hub page.</t>
         </is>
       </c>
     </row>
@@ -6182,19 +6182,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Kitchen Backsplash</t>
+          <t>Kitchen Islands</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>kitchen backsplash</t>
+          <t>kitchen island</t>
         </is>
       </c>
       <c r="E24" s="3" t="n">
-        <v>27100</v>
-      </c>
-      <c r="F24" s="6" t="n">
-        <v>44</v>
+        <v>90500</v>
+      </c>
+      <c r="F24" s="8" t="n">
+        <v>61</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -6208,7 +6208,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>High-demand feature page.</t>
+          <t>Highest demand of all (90.5K); high KD. Feature page funneling to remodels.</t>
         </is>
       </c>
     </row>
@@ -6220,42 +6220,38 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Service Area</t>
+          <t>Component</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Weddington, NC</t>
+          <t>Kitchen Backsplash</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>kitchen remodeling weddington nc</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F25" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
+          <t>kitchen backsplash ideas</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>18100</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>28</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="H25" s="10" t="inlineStr">
-        <is>
-          <t>Have — optimize</t>
+          <t>Buyer</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>New</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Page EXISTS.</t>
+          <t>Retarget to 'backsplash ideas' (KD 28) over generic 'kitchen backsplash' (KD 44).</t>
         </is>
       </c>
     </row>
@@ -6272,16 +6268,18 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Fort Mill, SC</t>
+          <t>Weddington, NC</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>kitchen remodeling fort mill sc</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="n">
-        <v>10</v>
+          <t>kitchen remodeling weddington nc</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
         <is>
@@ -6293,14 +6291,14 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="H26" s="10" t="inlineStr">
+      <c r="H26" s="11" t="inlineStr">
         <is>
           <t>Have — optimize</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Page EXISTS. SC side of the metro.</t>
+          <t>Page EXISTS.</t>
         </is>
       </c>
     </row>
@@ -6317,35 +6315,80 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
+          <t>Fort Mill, SC</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>kitchen remodeling fort mill sc</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="H27" s="11" t="inlineStr">
+        <is>
+          <t>Have — optimize</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Page EXISTS. SC side of the metro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Service Area</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
           <t>Huntersville / Mooresville / Belmont / +18 more</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>kitchen remodeling &lt;suburb&gt; nc</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="F27" s="12" t="inlineStr">
+      <c r="F28" s="12" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
       </c>
-      <c r="H27" s="10" t="inlineStr">
+      <c r="H28" s="11" t="inlineStr">
         <is>
           <t>Have — optimize</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>26 suburb pages EXIST total. The work is RANKING them via linked content, not building new ones.</t>
         </is>
@@ -6504,7 +6547,7 @@
       <c r="F4" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="G4" s="10" t="inlineStr">
+      <c r="G4" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -6537,9 +6580,9 @@
       <c r="F5" s="6" t="n">
         <v>48</v>
       </c>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -6636,7 +6679,7 @@
       <c r="F8" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="G8" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -6669,7 +6712,7 @@
       <c r="F9" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="G9" s="10" t="inlineStr">
+      <c r="G9" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -6966,7 +7009,7 @@
       <c r="F18" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="G18" s="10" t="inlineStr">
+      <c r="G18" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7032,7 +7075,7 @@
       <c r="F20" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G20" s="10" t="inlineStr">
+      <c r="G20" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7044,7 +7087,7 @@
           <t>kitchen remodeler</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -7065,7 +7108,7 @@
       <c r="F21" s="6" t="n">
         <v>48</v>
       </c>
-      <c r="G21" s="10" t="inlineStr">
+      <c r="G21" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7077,7 +7120,7 @@
           <t>kitchen remodel timeline</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -7197,7 +7240,7 @@
       <c r="F25" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G25" s="10" t="inlineStr">
+      <c r="G25" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7230,9 +7273,9 @@
       <c r="F26" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="G26" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -7362,7 +7405,7 @@
       <c r="F30" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="G30" s="10" t="inlineStr">
+      <c r="G30" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7428,7 +7471,7 @@
       <c r="F32" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="G32" s="10" t="inlineStr">
+      <c r="G32" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7560,7 +7603,7 @@
       <c r="F36" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="G36" s="10" t="inlineStr">
+      <c r="G36" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7626,9 +7669,9 @@
       <c r="F38" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="G38" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -7659,7 +7702,7 @@
       <c r="F39" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G39" s="10" t="inlineStr">
+      <c r="G39" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7692,9 +7735,9 @@
       <c r="F40" s="6" t="n">
         <v>48</v>
       </c>
-      <c r="G40" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -7704,7 +7747,7 @@
           <t>how long does a kitchen remodel take</t>
         </is>
       </c>
-      <c r="B41" s="8" t="inlineStr">
+      <c r="B41" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -7758,7 +7801,7 @@
       <c r="F42" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G42" s="10" t="inlineStr">
+      <c r="G42" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -7791,9 +7834,9 @@
       <c r="F43" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G43" s="11" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -7989,7 +8032,7 @@
       <c r="F49" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="G49" s="10" t="inlineStr">
+      <c r="G49" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -8055,7 +8098,7 @@
       <c r="F51" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G51" s="10" t="inlineStr">
+      <c r="G51" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -8385,7 +8428,7 @@
       <c r="F61" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G61" s="10" t="inlineStr">
+      <c r="G61" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -8418,7 +8461,7 @@
       <c r="F62" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="G62" s="10" t="inlineStr">
+      <c r="G62" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -8484,9 +8527,9 @@
       <c r="F64" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="G64" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -8517,9 +8560,9 @@
       <c r="F65" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="G65" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -8562,7 +8605,7 @@
           <t>how long does a kitchen renovation take</t>
         </is>
       </c>
-      <c r="B67" s="8" t="inlineStr">
+      <c r="B67" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -8616,9 +8659,9 @@
       <c r="F68" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="G68" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -8628,7 +8671,7 @@
           <t>kitchen contractor</t>
         </is>
       </c>
-      <c r="B69" s="8" t="inlineStr">
+      <c r="B69" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -8649,9 +8692,9 @@
       <c r="F69" s="6" t="n">
         <v>48</v>
       </c>
-      <c r="G69" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -8694,7 +8737,7 @@
           <t>kitchen remodel process</t>
         </is>
       </c>
-      <c r="B71" s="8" t="inlineStr">
+      <c r="B71" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -8814,9 +8857,9 @@
       <c r="F74" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="G74" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -8979,9 +9022,9 @@
       <c r="F79" s="6" t="n">
         <v>48</v>
       </c>
-      <c r="G79" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -9111,7 +9154,7 @@
       <c r="F83" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="G83" s="10" t="inlineStr">
+      <c r="G83" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -9123,7 +9166,7 @@
           <t>kitchen renovation timeline</t>
         </is>
       </c>
-      <c r="B84" s="8" t="inlineStr">
+      <c r="B84" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -9144,7 +9187,7 @@
       <c r="F84" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="G84" s="10" t="inlineStr">
+      <c r="G84" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -9156,7 +9199,7 @@
           <t>kitchen remodeling contractor</t>
         </is>
       </c>
-      <c r="B85" s="8" t="inlineStr">
+      <c r="B85" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -9210,7 +9253,7 @@
       <c r="F86" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G86" s="10" t="inlineStr">
+      <c r="G86" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -9243,7 +9286,7 @@
       <c r="F87" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G87" s="10" t="inlineStr">
+      <c r="G87" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -9474,9 +9517,9 @@
       <c r="F94" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G94" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -9540,7 +9583,7 @@
       <c r="F96" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G96" s="10" t="inlineStr">
+      <c r="G96" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -9552,7 +9595,7 @@
           <t>kitchen remodel order of steps</t>
         </is>
       </c>
-      <c r="B97" s="8" t="inlineStr">
+      <c r="B97" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -9573,9 +9616,9 @@
       <c r="F97" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G97" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -9684,7 +9727,7 @@
           <t>how long for a kitchen remodel</t>
         </is>
       </c>
-      <c r="B101" s="8" t="inlineStr">
+      <c r="B101" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -9738,7 +9781,7 @@
       <c r="F102" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G102" s="10" t="inlineStr">
+      <c r="G102" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -10068,9 +10111,9 @@
       <c r="F112" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="G112" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -10101,7 +10144,7 @@
       <c r="F113" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G113" s="10" t="inlineStr">
+      <c r="G113" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -10200,7 +10243,7 @@
       <c r="F116" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G116" s="10" t="inlineStr">
+      <c r="G116" s="11" t="inlineStr">
         <is>
           <t>Yes (planned)</t>
         </is>
@@ -10233,9 +10276,9 @@
       <c r="F117" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="G117" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -10365,9 +10408,9 @@
       <c r="F121" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="G121" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -10971,7 +11014,7 @@
           <t>remodeler</t>
         </is>
       </c>
-      <c r="B140" s="8" t="inlineStr">
+      <c r="B140" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -11103,7 +11146,7 @@
           <t>kitchen remodel timeline denver</t>
         </is>
       </c>
-      <c r="B144" s="8" t="inlineStr">
+      <c r="B144" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -11136,7 +11179,7 @@
           <t>kitchen remodeler davidson</t>
         </is>
       </c>
-      <c r="B145" s="8" t="inlineStr">
+      <c r="B145" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -11157,9 +11200,9 @@
       <c r="F145" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="G145" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -11400,7 +11443,7 @@
           <t>kitchen remodeler gastonia</t>
         </is>
       </c>
-      <c r="B153" s="8" t="inlineStr">
+      <c r="B153" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -11421,9 +11464,9 @@
       <c r="F153" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="G153" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -14061,9 +14104,9 @@
       <c r="F233" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G233" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -14193,9 +14236,9 @@
       <c r="F237" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G237" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -14226,9 +14269,9 @@
       <c r="F238" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G238" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -14259,9 +14302,9 @@
       <c r="F239" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G239" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -14292,9 +14335,9 @@
       <c r="F240" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G240" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -14325,9 +14368,9 @@
       <c r="F241" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G241" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -14457,9 +14500,9 @@
       <c r="F245" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G245" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -14490,9 +14533,9 @@
       <c r="F246" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G246" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -14523,9 +14566,9 @@
       <c r="F247" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G247" s="10" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -15393,7 +15436,7 @@
           <t>bathroom contractors</t>
         </is>
       </c>
-      <c r="B274" s="8" t="inlineStr">
+      <c r="B274" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -15855,7 +15898,7 @@
           <t>bathroom remodel contractors</t>
         </is>
       </c>
-      <c r="B288" s="8" t="inlineStr">
+      <c r="B288" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -15921,7 +15964,7 @@
           <t>bathroom remodel general contractor</t>
         </is>
       </c>
-      <c r="B290" s="8" t="inlineStr">
+      <c r="B290" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>
@@ -16482,7 +16525,7 @@
           <t>bathroom renovation contractors</t>
         </is>
       </c>
-      <c r="B307" s="8" t="inlineStr">
+      <c r="B307" s="9" t="inlineStr">
         <is>
           <t>Process &amp; Planning</t>
         </is>

</xml_diff>

<commit_message>
7 Day Kitchens: content-plan demand shown as local (Charlotte metro), not national
Selection still uses real national SEMrush volumes; DISPLAY now shows estimated
local demand (geo/GSC terms as-is; national topics scaled to Charlotte metro
share). Slide 11 + month headers relabeled "est. local demand" (~16K, matches
TJ's on-call framing) instead of 582K national.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/7-day-kitchens/keyword-research.xlsx
+++ b/decks/7-day-kitchens/keyword-research.xlsx
@@ -1031,7 +1031,7 @@
         </is>
       </c>
       <c r="G13" s="3" t="n">
-        <v>880</v>
+        <v>15</v>
       </c>
       <c r="H13" s="4" t="n">
         <v>4</v>
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="G15" s="3" t="n">
-        <v>1600</v>
+        <v>15</v>
       </c>
       <c r="H15" s="6" t="n">
         <v>44</v>
@@ -1145,7 +1145,7 @@
         </is>
       </c>
       <c r="G16" s="3" t="n">
-        <v>880</v>
+        <v>15</v>
       </c>
       <c r="H16" s="4" t="n">
         <v>25</v>
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="G21" s="3" t="n">
-        <v>33100</v>
+        <v>199</v>
       </c>
       <c r="H21" s="4" t="n">
         <v>23</v>
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="G22" s="3" t="n">
-        <v>90500</v>
+        <v>543</v>
       </c>
       <c r="H22" s="8" t="n">
         <v>52</v>
@@ -1411,7 +1411,7 @@
         </is>
       </c>
       <c r="G23" s="3" t="n">
-        <v>18100</v>
+        <v>109</v>
       </c>
       <c r="H23" s="4" t="n">
         <v>28</v>
@@ -1449,7 +1449,7 @@
         </is>
       </c>
       <c r="G24" s="3" t="n">
-        <v>12100</v>
+        <v>73</v>
       </c>
       <c r="H24" s="6" t="n">
         <v>40</v>
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="G25" s="3" t="n">
-        <v>3600</v>
+        <v>22</v>
       </c>
       <c r="H25" s="6" t="n">
         <v>34</v>
@@ -1525,7 +1525,7 @@
         </is>
       </c>
       <c r="G26" s="3" t="n">
-        <v>2400</v>
+        <v>15</v>
       </c>
       <c r="H26" s="6" t="n">
         <v>48</v>
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="G34" s="3" t="n">
-        <v>2900</v>
+        <v>17</v>
       </c>
       <c r="H34" s="8" t="n">
         <v>52</v>
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="G52" s="3" t="n">
-        <v>2900</v>
+        <v>17</v>
       </c>
       <c r="H52" s="4" t="n">
         <v>21</v>
@@ -2665,7 +2665,7 @@
         </is>
       </c>
       <c r="G56" s="3" t="n">
-        <v>880</v>
+        <v>15</v>
       </c>
       <c r="H56" s="6" t="n">
         <v>34</v>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="G62" s="3" t="n">
-        <v>40500</v>
+        <v>243</v>
       </c>
       <c r="H62" s="6" t="n">
         <v>44</v>
@@ -2931,7 +2931,7 @@
         </is>
       </c>
       <c r="G63" s="3" t="n">
-        <v>18100</v>
+        <v>109</v>
       </c>
       <c r="H63" s="6" t="n">
         <v>44</v>
@@ -2969,7 +2969,7 @@
         </is>
       </c>
       <c r="G64" s="3" t="n">
-        <v>12100</v>
+        <v>73</v>
       </c>
       <c r="H64" s="6" t="n">
         <v>30</v>
@@ -3007,7 +3007,7 @@
         </is>
       </c>
       <c r="G65" s="3" t="n">
-        <v>2900</v>
+        <v>17</v>
       </c>
       <c r="H65" s="8" t="n">
         <v>52</v>
@@ -3045,7 +3045,7 @@
         </is>
       </c>
       <c r="G66" s="3" t="n">
-        <v>2400</v>
+        <v>15</v>
       </c>
       <c r="H66" s="4" t="n">
         <v>26</v>
@@ -3349,7 +3349,7 @@
         </is>
       </c>
       <c r="G74" s="3" t="n">
-        <v>2400</v>
+        <v>15</v>
       </c>
       <c r="H74" s="8" t="n">
         <v>53</v>
@@ -3501,7 +3501,7 @@
         </is>
       </c>
       <c r="G78" s="3" t="n">
-        <v>880</v>
+        <v>15</v>
       </c>
       <c r="H78" s="6" t="n">
         <v>40</v>
@@ -4033,7 +4033,7 @@
         </is>
       </c>
       <c r="G92" s="3" t="n">
-        <v>2900</v>
+        <v>17</v>
       </c>
       <c r="H92" s="4" t="n">
         <v>20</v>
@@ -4147,7 +4147,7 @@
         </is>
       </c>
       <c r="G95" s="3" t="n">
-        <v>1900</v>
+        <v>15</v>
       </c>
       <c r="H95" s="6" t="n">
         <v>40</v>
@@ -4185,7 +4185,7 @@
         </is>
       </c>
       <c r="G96" s="3" t="n">
-        <v>880</v>
+        <v>15</v>
       </c>
       <c r="H96" s="6" t="n">
         <v>30</v>
@@ -4299,7 +4299,7 @@
         </is>
       </c>
       <c r="G99" s="3" t="n">
-        <v>165000</v>
+        <v>990</v>
       </c>
       <c r="H99" s="8" t="n">
         <v>55</v>
@@ -4337,7 +4337,7 @@
         </is>
       </c>
       <c r="G100" s="3" t="n">
-        <v>90500</v>
+        <v>543</v>
       </c>
       <c r="H100" s="4" t="n">
         <v>28</v>
@@ -4375,7 +4375,7 @@
         </is>
       </c>
       <c r="G101" s="3" t="n">
-        <v>33100</v>
+        <v>199</v>
       </c>
       <c r="H101" s="6" t="n">
         <v>48</v>
@@ -4413,7 +4413,7 @@
         </is>
       </c>
       <c r="G102" s="3" t="n">
-        <v>14800</v>
+        <v>89</v>
       </c>
       <c r="H102" s="6" t="n">
         <v>40</v>
@@ -4451,7 +4451,7 @@
         </is>
       </c>
       <c r="G103" s="3" t="n">
-        <v>9900</v>
+        <v>59</v>
       </c>
       <c r="H103" s="6" t="n">
         <v>41</v>
@@ -4489,7 +4489,7 @@
         </is>
       </c>
       <c r="G104" s="3" t="n">
-        <v>2900</v>
+        <v>17</v>
       </c>
       <c r="H104" s="4" t="n">
         <v>28</v>
@@ -17379,7 +17379,7 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>Demand/mo blends two verified sources: SEMrush search volume for the local commercial terms, and your own Google Search Console monthly impressions for everything you already appear for. Both are real, not estimates.</t>
+          <t>Demand/mo estimates monthly LOCAL (Charlotte-metro) demand: real local search volume for geo/commercial terms and your GSC impressions where you already appear, with national topic volumes scaled to Charlotte's metro share. The underlying national volumes (see the service-page tab) drove which articles to prioritize.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
7 Day Kitchens growth roadmap: rebuild deck + workbook off final content plan
Regenerated from the cleaned content plan (final titles, local demand 9,183,
PERPILLAR 18/52/10/40). Deck 16 slides, div-balanced/PASS. Workbook synced to
the live Google Sheet in place.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/7-day-kitchens/keyword-research.xlsx
+++ b/decks/7-day-kitchens/keyword-research.xlsx
@@ -627,12 +627,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling in Matthews, NC: What to Expect</t>
+          <t>Kitchen Remodeling in Waxhaw, NC: Local Process and Timeline</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>kitchen remodeling matthews nc</t>
+          <t>kitchen remodeling waxhaw nc</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -651,10 +651,10 @@
         </is>
       </c>
       <c r="G3" s="3" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -665,12 +665,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling in Huntersville, NC: Costs, Timelines, and Local Style</t>
+          <t>Kitchen Design Charlotte NC: One Local Crew, Start to Finish</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>kitchen remodeling huntersville nc</t>
+          <t>kitchen design charlotte nc</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="G4" s="3" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="H4" s="4" t="n">
         <v>18</v>
@@ -703,12 +703,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Charlotte Kitchen Renovation: A Faster, Fixed-Price Approach</t>
+          <t>Kitchen Remodeling in Denver, NC: West Lake Norman Kitchens</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>charlotte kitchen renovation</t>
+          <t>kitchen remodeling denver nc</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -727,10 +727,10 @@
         </is>
       </c>
       <c r="G5" s="3" t="n">
-        <v>320</v>
+        <v>10</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -741,12 +741,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Kitchen Designers Charlotte: What the Process Looks Like Here</t>
+          <t>Kitchen Remodel in Charlotte, NC: Fixed Pricing, Done in 7 Days</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>kitchen designers charlotte</t>
+          <t>kitchen remodel charlotte nc</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -765,10 +765,10 @@
         </is>
       </c>
       <c r="G6" s="3" t="n">
-        <v>153</v>
+        <v>390</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7">
@@ -779,7 +779,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling Company Charlotte: Where Speed Meets Craftsmanship</t>
+          <t>Kitchen Remodeling Company Charlotte: What the Process Looks Like Here</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -817,12 +817,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling Companies Charlotte: Local Crews, Lifetime Warranty</t>
+          <t>Kitchen Remodeling in Tega Cay, SC: Lakefront Kitchen Renovations</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>kitchen remodeling companies charlotte</t>
+          <t>kitchen remodeling tega cay sc</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -841,10 +841,10 @@
         </is>
       </c>
       <c r="G8" s="3" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
@@ -855,12 +855,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kitchen and Bath Remodeling in Charlotte, NC: One Crew, One Timeline</t>
+          <t>Custom Kitchen Remodels in Charlotte: Built Around Your Space</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>kitchen and bath remodeling charlotte nc</t>
+          <t>custom kitchen remodel charlotte</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -879,10 +879,10 @@
         </is>
       </c>
       <c r="G9" s="3" t="n">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10">
@@ -893,12 +893,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling in Concord, NC: A Local Renovation Guide</t>
+          <t>Kitchen Remodeling in Belmont, NC: Local Trends and Timelines</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>kitchen remodeling concord nc</t>
+          <t>kitchen remodeling belmont nc</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -917,10 +917,10 @@
         </is>
       </c>
       <c r="G10" s="3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11">
@@ -931,12 +931,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling in Indian Trail, NC: Costs and What to Expect</t>
+          <t>Kitchen Remodel Providence Plantation NC: Fixed Pricing, Finished in 7 Days</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>kitchen remodeling indian trail nc</t>
+          <t>kitchen remodel providence plantation nc</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -955,7 +955,7 @@
         </is>
       </c>
       <c r="G11" s="3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H11" s="4" t="n">
         <v>18</v>
@@ -969,17 +969,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Why a Fixed-Price Kitchen Remodel Beats Hourly Surprises</t>
+          <t>Ballantyne Kitchen Remodeling: Premium Results Without the Wait</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>fixed price kitchen remodel</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Cost &amp; Budget</t>
+          <t>kitchen remodeling ballantyne</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Charlotte &amp; Local</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -993,10 +993,10 @@
         </is>
       </c>
       <c r="G12" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H12" s="6" t="n">
-        <v>30</v>
+        <v>10</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="13">
@@ -1007,22 +1007,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Quartz Countertop Pricing: What Sets the Range</t>
+          <t>Kitchen Remodeling in Fort Mill, SC: What Local Homeowners Should Know</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>quartz price</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Cost &amp; Budget</t>
+          <t>kitchen remodeling fort mill sc</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Charlotte &amp; Local</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1031,10 +1031,10 @@
         </is>
       </c>
       <c r="G13" s="3" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14">
@@ -1045,22 +1045,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>The Average Cost of a Kitchen Remodel, and Why Yours May Differ</t>
+          <t>Custom Kitchen Cabinets in Charlotte: Built for Your Space</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>average cost of kitchen remodel</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Cost &amp; Budget</t>
+          <t>custom kitchen cabinets charlotte</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Charlotte &amp; Local</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1083,22 +1083,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>How to Set a Kitchen Remodel Budget You Won't Blow Through</t>
+          <t>Affordable Kitchen Remodel Charlotte NC: Built Around Your Home and Budget</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>kitchen remodel budget</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Cost &amp; Budget</t>
+          <t>affordable kitchen remodel charlotte nc</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Charlotte &amp; Local</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1107,10 +1107,10 @@
         </is>
       </c>
       <c r="G15" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="H15" s="6" t="n">
-        <v>44</v>
+        <v>10</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="16">
@@ -1121,12 +1121,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>What a Kitchen Island Costs to Build In</t>
+          <t>Why a Fixed-Price Kitchen Remodel Beats Hourly Surprises</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>kitchen island cost</t>
+          <t>fixed price kitchen remodel</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -1136,19 +1136,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G16" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="H16" s="4" t="n">
-        <v>25</v>
+        <v>40</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="17">
@@ -1159,12 +1159,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Budget Backsplash Ideas That Still Look High-End</t>
+          <t>What Quartz Countertops Cost, Installed</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>cheap backsplash</t>
+          <t>cost of quartz countertops</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -1183,10 +1183,10 @@
         </is>
       </c>
       <c r="G17" s="3" t="n">
-        <v>480</v>
+        <v>17</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18">
@@ -1197,12 +1197,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Budget-Friendly Kitchen Remodels: Smart Places to Save</t>
+          <t>Small Kitchen Remodels: Where the Budget Goes</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>budget friendly kitchen remodel</t>
+          <t>small kitchen remodel price</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -1221,10 +1221,10 @@
         </is>
       </c>
       <c r="G18" s="3" t="n">
-        <v>320</v>
-      </c>
-      <c r="H18" s="6" t="n">
-        <v>33</v>
+        <v>480</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="19">
@@ -1235,12 +1235,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Choosing Backsplash Prices Without Regret</t>
+          <t>Laminate Countertops: The Budget-Friendly Counter Option</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>backsplash prices</t>
+          <t>laminate countertop cost</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -1259,10 +1259,10 @@
         </is>
       </c>
       <c r="G19" s="3" t="n">
-        <v>140</v>
+        <v>15</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20">
@@ -1273,12 +1273,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Financing a Kitchen Remodel: Options Weighed Honestly</t>
+          <t>Backsplash Prices, Weighed Honestly</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>kitchen remodel financing</t>
+          <t>backsplash prices</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -1297,10 +1297,10 @@
         </is>
       </c>
       <c r="G20" s="3" t="n">
-        <v>10</v>
+        <v>140</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21">
@@ -1311,12 +1311,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Peel-and-Stick Backsplash: Quick Fix or False Economy?</t>
+          <t>Cabinet Refacing in Charlotte, NC: When It Makes Sense</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>peel and stick backsplash</t>
+          <t>cabinet refacing charlotte nc</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1335,10 +1335,10 @@
         </is>
       </c>
       <c r="G21" s="3" t="n">
-        <v>199</v>
+        <v>102</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22">
@@ -1349,12 +1349,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Should Your Kitchen Have an Island? A Layout Guide</t>
+          <t>Peel and Stick Tile Backsplash: The Trade-offs That Matter</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>kitchen island</t>
+          <t>peel and stick tile backsplash</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -1373,10 +1373,10 @@
         </is>
       </c>
       <c r="G22" s="3" t="n">
-        <v>543</v>
-      </c>
-      <c r="H22" s="8" t="n">
-        <v>52</v>
+        <v>32</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="23">
@@ -1387,12 +1387,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Kitchen Backsplash Ideas That Pull a Remodel Together</t>
+          <t>Quartz Countertops: Why They Dominate Modern Kitchens</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>kitchen backsplash ideas</t>
+          <t>quartz countertops</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -1402,16 +1402,16 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G23" s="3" t="n">
-        <v>109</v>
+        <v>543</v>
       </c>
       <c r="H23" s="4" t="n">
         <v>28</v>
@@ -1425,12 +1425,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Kitchen Island Ideas: Sizing, Seating, and Smart Storage</t>
+          <t>Kitchen Countertops Compared: Quartz, Granite, and the Alternatives</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>kitchen island ideas</t>
+          <t>kitchen countertops</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -1440,19 +1440,19 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G24" s="3" t="n">
-        <v>73</v>
+        <v>199</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25">
@@ -1463,12 +1463,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Galley Kitchen Ideas: Big Function in a Narrow Footprint</t>
+          <t>Adding a Scullery to Your Kitchen: The Hidden Prep-Space Trend</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>galley kitchen ideas</t>
+          <t>kitchen scullery</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -1483,14 +1483,14 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G25" s="3" t="n">
-        <v>22</v>
+        <v>109</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>34</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26">
@@ -1501,12 +1501,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Open-Concept Kitchens: When Knocking Down a Wall Pays Off</t>
+          <t>Kitchen Island Ideas: Sizing, Seating, and Smart Storage</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>open concept kitchen</t>
+          <t>kitchen island ideas</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -1521,14 +1521,14 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G26" s="3" t="n">
-        <v>15</v>
+        <v>73</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27">
@@ -1539,12 +1539,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Kitchen Layout Basics: Work Triangles, Walkways, and Flow</t>
+          <t>Kitchen Tile: Floor, Backsplash, and Where Each Works</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>kitchen layout</t>
+          <t>kitchen tile</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1566,7 +1566,7 @@
         <v>40</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>48</v>
+        <v>31</v>
       </c>
     </row>
     <row r="28">
@@ -1577,12 +1577,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Kitchen Lighting Ideas: Layering Task, Ambient, and Accent</t>
+          <t>Kitchen Accessories: What to Know Before You Commit</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>kitchen lighting ideas</t>
+          <t>kitchen accessories</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -1592,19 +1592,19 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G28" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="H28" s="6" t="n">
-        <v>38</v>
+      <c r="H28" s="8" t="n">
+        <v>52</v>
       </c>
     </row>
     <row r="29">
@@ -1615,12 +1615,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Modern Kitchen Design: Clean Lines Without the Cold Feel</t>
+          <t>Kitchen Bars and Breakfast Counters: Seating That Works</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>modern kitchen design</t>
+          <t>kitchen bar</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1639,10 +1639,10 @@
         </is>
       </c>
       <c r="G29" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="H29" s="6" t="n">
         <v>40</v>
-      </c>
-      <c r="H29" s="6" t="n">
-        <v>38</v>
       </c>
     </row>
     <row r="30">
@@ -1653,12 +1653,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Pantry Ideas: Designing Storage That Earns Its Footprint</t>
+          <t>Kitchen Storage Ideas That Use Every Inch</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>pantry ideas</t>
+          <t>kitchen storage ideas</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
@@ -1677,10 +1677,10 @@
         </is>
       </c>
       <c r="G30" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H30" s="6" t="n">
-        <v>48</v>
+        <v>17</v>
+      </c>
+      <c r="H30" s="8" t="n">
+        <v>52</v>
       </c>
     </row>
     <row r="31">
@@ -1691,12 +1691,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Two-Tone Kitchen Cabinets: How to Mix Without a Mess</t>
+          <t>Kitchen Cabinet Styles: Shaker, Flat-Panel, and Beyond</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>two tone kitchen cabinets</t>
+          <t>kitchen cabinet styles</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
@@ -1715,10 +1715,10 @@
         </is>
       </c>
       <c r="G31" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H31" s="6" t="n">
-        <v>30</v>
+        <v>15</v>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="32">
@@ -1729,12 +1729,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Walk-In Pantry Ideas for Your Kitchen Remodel</t>
+          <t>Kitchen Remodel Before and After: What a Week Can Change</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>walk in pantry ideas</t>
+          <t>kitchen remodel before and after</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="G32" s="3" t="n">
-        <v>40</v>
+        <v>590</v>
       </c>
       <c r="H32" s="6" t="n">
         <v>30</v>
@@ -1767,22 +1767,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Kitchen Remodel Contractors in Rock Hill, SC</t>
+          <t>Quartz vs Granite Countertops: Which Wins for Your Kitchen</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>contractor for kitchen remodel rock hill sc</t>
-        </is>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
-        <is>
-          <t>Process &amp; Planning</t>
+          <t>quartz vs granite</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1791,10 +1791,10 @@
         </is>
       </c>
       <c r="G33" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H33" s="4" t="n">
-        <v>24</v>
+        <v>40</v>
+      </c>
+      <c r="H33" s="6" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="34">
@@ -1805,22 +1805,22 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Kitchen Renovation Contractors: What to Expect, Day by Day</t>
+          <t>Kitchen Flooring Options Ranked for Durability and Looks</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>kitchen renovation contractors</t>
-        </is>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
-        <is>
-          <t>Process &amp; Planning</t>
+          <t>kitchen flooring options</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1829,10 +1829,10 @@
         </is>
       </c>
       <c r="G34" s="3" t="n">
-        <v>17</v>
-      </c>
-      <c r="H34" s="8" t="n">
-        <v>52</v>
+        <v>40</v>
+      </c>
+      <c r="H34" s="6" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="35">
@@ -1843,34 +1843,34 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Bathroom and Kitchen Contractors: What Separates Great From Cheap</t>
+          <t>Farmhouse Kitchen Ideas That Still Feel Fresh in 2026</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>bathroom and kitchen contractors</t>
-        </is>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
-        <is>
-          <t>Process &amp; Planning</t>
+          <t>farmhouse kitchen ideas</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G35" s="3" t="n">
-        <v>390</v>
+        <v>40</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
     </row>
     <row r="36">
@@ -1881,22 +1881,22 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>DIY Kitchen Furniture: The Process, Demystified</t>
+          <t>Choosing a Kitchen Faucet: Finishes, Features, and Value</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>diy kitchen furniture</t>
-        </is>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>Process &amp; Planning</t>
+          <t>kitchen faucet ideas</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1905,10 +1905,10 @@
         </is>
       </c>
       <c r="G36" s="3" t="n">
-        <v>390</v>
-      </c>
-      <c r="H36" s="4" t="n">
-        <v>23</v>
+        <v>40</v>
+      </c>
+      <c r="H36" s="6" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="37">
@@ -1919,22 +1919,22 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Tiny Kitchen Plans: Timelines, Trade-offs, and Questions to Ask</t>
+          <t>Cabinet Hardware: The Small Detail That Sets the Tone</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>tiny kitchen plans</t>
-        </is>
-      </c>
-      <c r="D37" s="9" t="inlineStr">
-        <is>
-          <t>Process &amp; Planning</t>
+          <t>cabinet hardware ideas</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1943,10 +1943,10 @@
         </is>
       </c>
       <c r="G37" s="3" t="n">
-        <v>320</v>
-      </c>
-      <c r="H37" s="4" t="n">
-        <v>20</v>
+        <v>40</v>
+      </c>
+      <c r="H37" s="6" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="38">
@@ -1957,17 +1957,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Small Kitchen Plans: What Every Remodel Should Know</t>
+          <t>Butler's Pantry Ideas: A Kitchen Upgrade That Adds Real Value</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>small kitchen plans</t>
-        </is>
-      </c>
-      <c r="D38" s="9" t="inlineStr">
-        <is>
-          <t>Process &amp; Planning</t>
+          <t>butler pantry ideas</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="G38" s="3" t="n">
-        <v>170</v>
-      </c>
-      <c r="H38" s="4" t="n">
-        <v>15</v>
+        <v>40</v>
+      </c>
+      <c r="H38" s="6" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="39">
@@ -1995,12 +1995,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Open Kitchen Living Room: Timelines, Trade-offs, and Questions to Ask</t>
+          <t>How to Plan a Kitchen Remodel Before Demo Day</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>open kitchen living room</t>
+          <t>how to plan a kitchen remodel</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
@@ -2010,7 +2010,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2019,10 +2019,10 @@
         </is>
       </c>
       <c r="G39" s="3" t="n">
-        <v>720</v>
+        <v>40</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="40">
@@ -2033,12 +2033,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>The Kitchen Remodel Checklist Every Homeowner Should Use</t>
+          <t>Do You Need a Permit for a Kitchen Remodel in North Carolina?</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>kitchen remodel checklist</t>
+          <t>kitchen remodel permits</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G40" s="3" t="n">
@@ -2071,12 +2071,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling Timeline: What It Takes, Start to Finish</t>
+          <t>Change Orders on a Kitchen Remodel: How Fixed Pricing Avoids Them</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>kitchen remodeling timeline</t>
+          <t>kitchen remodel change orders</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
@@ -2095,10 +2095,10 @@
         </is>
       </c>
       <c r="G41" s="3" t="n">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="H41" s="6" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
     </row>
     <row r="42">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Kitchen Design and Build Charlotte NC: A Faster Path to Your Dream Kitchen</t>
+          <t>Kitchen Design-Build in Charlotte, NC: One Team, Start to Finish</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2147,12 +2147,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling in Mooresville, NC: A Lake Norman Homeowner's Guide</t>
+          <t>Kitchen Remodeling in Matthews, NC: What to Expect</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>kitchen remodeling mooresville nc</t>
+          <t>kitchen remodeling matthews nc</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -2171,7 +2171,7 @@
         </is>
       </c>
       <c r="G43" s="3" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H43" s="4" t="n">
         <v>18</v>
@@ -2185,12 +2185,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>What Makes the Best Kitchen Contractor in Charlotte</t>
+          <t>Kitchen Contractor Belmont, Done the Fixed-Price Way</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>best kitchen contractor charlotte</t>
+          <t>kitchen contractor belmont</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2209,10 +2209,10 @@
         </is>
       </c>
       <c r="G44" s="3" t="n">
-        <v>90</v>
-      </c>
-      <c r="H44" s="6" t="n">
-        <v>30</v>
+        <v>15</v>
+      </c>
+      <c r="H44" s="4" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="45">
@@ -2223,12 +2223,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Charlotte Kitchen Remodeling: Fixed Pricing, Finished in 7 Days</t>
+          <t>Kitchen Remodeling in Lake Wylie, SC: What Local Homeowners Should Know</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>charlotte kitchen remodeling</t>
+          <t>kitchen remodeling lake wylie sc</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -2247,10 +2247,10 @@
         </is>
       </c>
       <c r="G45" s="3" t="n">
-        <v>320</v>
+        <v>10</v>
       </c>
       <c r="H45" s="4" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="46">
@@ -2261,12 +2261,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Hiring a Kitchen Contractor in Charlotte: A Vetting Guide</t>
+          <t>Kitchen Designers Charlotte: Fixed Pricing, Finished in 7 Days</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>kitchen contractor charlotte</t>
+          <t>kitchen designers charlotte</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2285,10 +2285,10 @@
         </is>
       </c>
       <c r="G46" s="3" t="n">
-        <v>90</v>
+        <v>153</v>
       </c>
       <c r="H46" s="4" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="47">
@@ -2299,12 +2299,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Best Kitchen Remodeler Charlotte: The 7-Day Difference, Explained</t>
+          <t>Kitchen Remodeling Services Charlotte: Built Around Your Home and Budget</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>best kitchen remodeler charlotte</t>
+          <t>kitchen remodeling services charlotte</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -2323,7 +2323,7 @@
         </is>
       </c>
       <c r="G47" s="3" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="H47" s="4" t="n">
         <v>18</v>
@@ -2337,12 +2337,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Kitchen Renovation Services Charlotte: What the Process Looks Like Here</t>
+          <t>Kitchen Remodeling South West Charlotte: A Faster Path to Your Dream Kitchen</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>kitchen renovation services charlotte</t>
+          <t>kitchen remodeling south west charlotte</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2361,10 +2361,10 @@
         </is>
       </c>
       <c r="G48" s="3" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="H48" s="4" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
     </row>
     <row r="49">
@@ -2375,12 +2375,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling South West Charlotte: One Local Crew, Start to Finish</t>
+          <t>High-End Kitchen Remodels in Charlotte: Premium, Fixed-Price</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>kitchen remodeling south west charlotte</t>
+          <t>high-end kitchen remodel charlotte</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -2399,10 +2399,10 @@
         </is>
       </c>
       <c r="G49" s="3" t="n">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="H49" s="4" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="50">
@@ -2413,12 +2413,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling in Fort Mill, SC: What Local Homeowners Should Know</t>
+          <t>Kitchen Remodeling in Concord, NC: A Local Renovation Guide</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>kitchen remodeling fort mill sc</t>
+          <t>kitchen remodeling concord nc</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -2437,7 +2437,7 @@
         </is>
       </c>
       <c r="G50" s="3" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H50" s="4" t="n">
         <v>18</v>
@@ -2451,12 +2451,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling in Mint Hill, NC: A Local Homeowner's Guide</t>
+          <t>Kitchen Remodel Raintree NC: Local Crews, Lifetime Warranty</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>kitchen remodeling mint hill nc</t>
+          <t>kitchen remodel raintree nc</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -2475,7 +2475,7 @@
         </is>
       </c>
       <c r="G51" s="3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H51" s="4" t="n">
         <v>18</v>
@@ -2489,22 +2489,22 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>What Quartz Countertops Cost, Installed</t>
+          <t>Kitchen Remodeling in Davidson, NC: A Lake Norman Town Guide</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>cost of quartz countertops</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Cost &amp; Budget</t>
+          <t>kitchen remodeling davidson nc</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Charlotte &amp; Local</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2513,10 +2513,10 @@
         </is>
       </c>
       <c r="G52" s="3" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="H52" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="53">
@@ -2527,34 +2527,34 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Small Kitchen Remodels: Where the Budget Goes</t>
+          <t>Kitchen Remodeling in Indian Trail, NC: Costs and What to Expect</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>small kitchen remodel price</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>Cost &amp; Budget</t>
+          <t>kitchen remodeling indian trail nc</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Charlotte &amp; Local</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G53" s="3" t="n">
-        <v>480</v>
+        <v>10</v>
       </c>
       <c r="H53" s="4" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="54">
@@ -2565,34 +2565,34 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>How Much Space to Leave Between Counter and Island</t>
+          <t>Cabinet Installation Charlotte NC: What the Process Looks Like Here</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>how much space between counter and island</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>Cost &amp; Budget</t>
+          <t>cabinet installation charlotte nc</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Charlotte &amp; Local</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G54" s="3" t="n">
-        <v>320</v>
+        <v>10</v>
       </c>
       <c r="H54" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="55">
@@ -2603,12 +2603,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Cheap Backsplash Options: What to Know Before You Commit</t>
+          <t>What Granite Countertops Cost, Installed</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>cheap backsplash options</t>
+          <t>cost of granite countertops</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
@@ -2627,10 +2627,10 @@
         </is>
       </c>
       <c r="G55" s="3" t="n">
-        <v>260</v>
+        <v>17</v>
       </c>
       <c r="H55" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="56">
@@ -2641,12 +2641,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Laminate Countertops: The Budget-Friendly Counter Option</t>
+          <t>What a Small Kitchen Remodel Really Costs</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>laminate countertop cost</t>
+          <t>average cost of small kitchen remodel</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
@@ -2661,14 +2661,14 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G56" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="H56" s="6" t="n">
-        <v>34</v>
+        <v>390</v>
+      </c>
+      <c r="H56" s="4" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="57">
@@ -2679,12 +2679,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>A Kitchen Makeover on a Budget: What's Realistic</t>
+          <t>The Average Cost of a Kitchen Remodel, and Why Yours May Differ</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>kitchen makeover on a budget</t>
+          <t>average cost of kitchen remodel</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
@@ -2699,14 +2699,14 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G57" s="3" t="n">
-        <v>390</v>
-      </c>
-      <c r="H57" s="6" t="n">
-        <v>32</v>
+        <v>10</v>
+      </c>
+      <c r="H57" s="4" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="58">
@@ -2717,12 +2717,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Small Kitchen Remodels on a Budget: What to Budget Before You Start</t>
+          <t>How to Set a Kitchen Remodel Budget You Won't Blow Through</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>small kitchen remodels on a budget</t>
+          <t>kitchen remodel budget</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
@@ -2741,10 +2741,10 @@
         </is>
       </c>
       <c r="G58" s="3" t="n">
-        <v>260</v>
-      </c>
-      <c r="H58" s="4" t="n">
-        <v>27</v>
+        <v>15</v>
+      </c>
+      <c r="H58" s="6" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="59">
@@ -2755,12 +2755,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Kitchen Renovation Cost: A Room-by-Room Money Map</t>
+          <t>Cheap Backsplash Ideas: A Plain-English Cost Primer</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>kitchen renovation cost</t>
+          <t>cheap backsplash ideas</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
@@ -2770,7 +2770,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2779,7 +2779,7 @@
         </is>
       </c>
       <c r="G59" s="3" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H59" s="6" t="n">
         <v>30</v>
@@ -2793,22 +2793,22 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Cabinet Refacing in Charlotte, NC: When It Makes Sense</t>
+          <t>Budget Backsplash Ideas That Still Look High-End</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>cabinet refacing charlotte nc</t>
-        </is>
-      </c>
-      <c r="D60" s="7" t="inlineStr">
-        <is>
-          <t>Design &amp; Materials</t>
+          <t>cheap backsplash</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Cost &amp; Budget</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2817,10 +2817,10 @@
         </is>
       </c>
       <c r="G60" s="3" t="n">
-        <v>102</v>
+        <v>480</v>
       </c>
       <c r="H60" s="4" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="61">
@@ -2831,22 +2831,22 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Kitchen and Laundry Room Combos: Designing the Two as One Project</t>
+          <t>Kitchen Renovation Cost: A Room-by-Room Money Map</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>kitchen and laundry room remodel</t>
-        </is>
-      </c>
-      <c r="D61" s="7" t="inlineStr">
-        <is>
-          <t>Design &amp; Materials</t>
+          <t>kitchen renovation cost</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Cost &amp; Budget</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2855,10 +2855,10 @@
         </is>
       </c>
       <c r="G61" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H61" s="4" t="n">
-        <v>24</v>
+        <v>60</v>
+      </c>
+      <c r="H61" s="6" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="62">
@@ -2869,17 +2869,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Butcher Block Countertops: Warm Looks, Real Trade-offs</t>
+          <t>Financing a Kitchen Remodel: Options Weighed Honestly</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>butcher block countertops</t>
-        </is>
-      </c>
-      <c r="D62" s="7" t="inlineStr">
-        <is>
-          <t>Design &amp; Materials</t>
+          <t>kitchen remodel financing</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Cost &amp; Budget</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2893,10 +2893,10 @@
         </is>
       </c>
       <c r="G62" s="3" t="n">
-        <v>243</v>
+        <v>10</v>
       </c>
       <c r="H62" s="6" t="n">
-        <v>44</v>
+        <v>30</v>
       </c>
     </row>
     <row r="63">
@@ -2907,12 +2907,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Adding a Scullery to Your Kitchen: The Hidden Prep-Space Trend</t>
+          <t>Choosing Kitchen Cabinets: Styles, Finishes, and What Lasts</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>kitchen scullery</t>
+          <t>kitchen cabinets</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -2931,10 +2931,10 @@
         </is>
       </c>
       <c r="G63" s="3" t="n">
-        <v>109</v>
-      </c>
-      <c r="H63" s="6" t="n">
-        <v>44</v>
+        <v>990</v>
+      </c>
+      <c r="H63" s="8" t="n">
+        <v>55</v>
       </c>
     </row>
     <row r="64">
@@ -2945,12 +2945,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Subway Tile Backsplash: The Timeless Default, Done Right</t>
+          <t>Stick on Backsplash: What to Weigh First</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>subway tile backsplash</t>
+          <t>stick on backsplash</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
@@ -2969,10 +2969,10 @@
         </is>
       </c>
       <c r="G64" s="3" t="n">
-        <v>73</v>
-      </c>
-      <c r="H64" s="6" t="n">
-        <v>30</v>
+        <v>26</v>
+      </c>
+      <c r="H64" s="4" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="65">
@@ -2983,12 +2983,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Kitchen Storage Ideas That Use Every Inch</t>
+          <t>Should Your Kitchen Have an Island? A Layout Guide</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>kitchen storage ideas</t>
+          <t>kitchen island</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
@@ -2998,16 +2998,16 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G65" s="3" t="n">
-        <v>17</v>
+        <v>543</v>
       </c>
       <c r="H65" s="8" t="n">
         <v>52</v>
@@ -3021,12 +3021,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Kitchen Cabinet Styles: Shaker, Flat-Panel, and Beyond</t>
+          <t>Kitchen Island with Seating: What Designers Pick and Why</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>kitchen cabinet styles</t>
+          <t>kitchen island with seating</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
@@ -3036,19 +3036,19 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G66" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="H66" s="4" t="n">
-        <v>26</v>
+        <v>163</v>
+      </c>
+      <c r="H66" s="6" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="67">
@@ -3059,12 +3059,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Kitchen Design Ideas: Layouts, Light, and Lasting Style</t>
+          <t>Kitchen Utensils: A Homeowner's Buyer Guide</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>kitchen design ideas</t>
+          <t>kitchen utensils</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3083,10 +3083,10 @@
         </is>
       </c>
       <c r="G67" s="3" t="n">
-        <v>40</v>
+        <v>109</v>
       </c>
       <c r="H67" s="6" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="68">
@@ -3097,12 +3097,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Kitchen Cabinet Colors: What's Timeless vs What's Trendy</t>
+          <t>Subway Tile Backsplash: The Timeless Default, Done Right</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>kitchen cabinet colors</t>
+          <t>subway tile backsplash</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
@@ -3112,7 +3112,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3121,10 +3121,10 @@
         </is>
       </c>
       <c r="G68" s="3" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="H68" s="6" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
     </row>
     <row r="69">
@@ -3135,12 +3135,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Kitchen Trends 2026: Bold Cabinets, Brass, and What to Skip</t>
+          <t>Kitchen Island with Storage: Weighed Honestly for Your Budget</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>kitchen trends 2026</t>
+          <t>kitchen island with storage</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
@@ -3150,19 +3150,19 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G69" s="3" t="n">
         <v>40</v>
       </c>
       <c r="H69" s="6" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="70">
@@ -3173,12 +3173,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Kitchen Sink Ideas: Materials, Mounts, and the Right Size</t>
+          <t>Choosing Kitchen and Bath Without Regret</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>kitchen sink ideas</t>
+          <t>kitchen and bath</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
@@ -3188,19 +3188,19 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G70" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H70" s="6" t="n">
-        <v>38</v>
+        <v>32</v>
+      </c>
+      <c r="H70" s="8" t="n">
+        <v>51</v>
       </c>
     </row>
     <row r="71">
@@ -3211,12 +3211,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Kitchen Paint Colors That Flatter Cabinets and Counters</t>
+          <t>Galley Kitchen Ideas: Big Function in a Narrow Footprint</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>kitchen paint colors</t>
+          <t>galley kitchen ideas</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
@@ -3231,14 +3231,14 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G71" s="3" t="n">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="H71" s="6" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="72">
@@ -3249,12 +3249,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Kitchen Appliances: Where to Splurge and Where to Save</t>
+          <t>Waterfall Islands: The Statement Feature Worth the Splurge</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>kitchen appliances</t>
+          <t>waterfall island</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3273,10 +3273,10 @@
         </is>
       </c>
       <c r="G72" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H72" s="6" t="n">
-        <v>48</v>
+        <v>17</v>
+      </c>
+      <c r="H72" s="4" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="73">
@@ -3287,12 +3287,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Kitchen and Mudroom Combos: A Smarter Family Entryway</t>
+          <t>Kitchen Layout Basics: Work Triangles, Walkways, and Flow</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>kitchen and mudroom</t>
+          <t>kitchen layout</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
@@ -3314,7 +3314,7 @@
         <v>40</v>
       </c>
       <c r="H73" s="6" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="74">
@@ -3325,34 +3325,34 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Kitchen Contractors: Done Right the First Time</t>
+          <t>Kitchen Lighting Ideas: Layering Task, Ambient, and Accent</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>kitchen contractors</t>
-        </is>
-      </c>
-      <c r="D74" s="9" t="inlineStr">
-        <is>
-          <t>Process &amp; Planning</t>
+          <t>kitchen lighting ideas</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G74" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="H74" s="8" t="n">
-        <v>53</v>
+        <v>40</v>
+      </c>
+      <c r="H74" s="6" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="75">
@@ -3363,22 +3363,22 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Local Kitchen Remodelers: The Questions to Ask First</t>
+          <t>Modern Kitchen Design: Clean Lines Without the Cold Feel</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>local kitchen remodelers</t>
-        </is>
-      </c>
-      <c r="D75" s="9" t="inlineStr">
-        <is>
-          <t>Process &amp; Planning</t>
+          <t>modern kitchen design</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3387,10 +3387,10 @@
         </is>
       </c>
       <c r="G75" s="3" t="n">
-        <v>320</v>
-      </c>
-      <c r="H75" s="8" t="n">
-        <v>50</v>
+        <v>40</v>
+      </c>
+      <c r="H75" s="6" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="76">
@@ -3401,34 +3401,34 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>How to Compare the Best Kitchen Remodel Contractors</t>
+          <t>Pantry Ideas: Designing Storage That Earns Its Footprint</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>best kitchen remodel contractors</t>
-        </is>
-      </c>
-      <c r="D76" s="9" t="inlineStr">
-        <is>
-          <t>Process &amp; Planning</t>
+          <t>pantry ideas</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G76" s="3" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="H76" s="6" t="n">
-        <v>30</v>
+        <v>48</v>
       </c>
     </row>
     <row r="77">
@@ -3439,17 +3439,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>How to Prepare Your Home for a Kitchen Remodel</t>
+          <t>Two-Tone Kitchen Cabinets: How to Mix Without a Mess</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>how to prepare for a kitchen remodel</t>
-        </is>
-      </c>
-      <c r="D77" s="9" t="inlineStr">
-        <is>
-          <t>Process &amp; Planning</t>
+          <t>two tone kitchen cabinets</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3459,14 +3459,14 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G77" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H77" s="4" t="n">
-        <v>24</v>
+        <v>40</v>
+      </c>
+      <c r="H77" s="6" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="78">
@@ -3477,17 +3477,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>DIY Kitchen Cupboards: A Homeowner's Walkthrough</t>
+          <t>Walk-In Pantry Ideas for Your Kitchen Remodel</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>diy kitchen cupboards</t>
-        </is>
-      </c>
-      <c r="D78" s="9" t="inlineStr">
-        <is>
-          <t>Process &amp; Planning</t>
+          <t>walk in pantry ideas</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3501,10 +3501,10 @@
         </is>
       </c>
       <c r="G78" s="3" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="H78" s="6" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="79">
@@ -3515,12 +3515,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Galley Kitchen Plans: How to Pick the Right Pro</t>
+          <t>Kitchen Remodel Contractors in Rock Hill, SC</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>galley kitchen plans</t>
+          <t>contractor for kitchen remodel rock hill sc</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
@@ -3530,19 +3530,19 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G79" s="3" t="n">
-        <v>720</v>
+        <v>10</v>
       </c>
       <c r="H79" s="4" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="80">
@@ -3553,12 +3553,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Kitchen Demolition: What Tear-Out Day Actually Involves</t>
+          <t>Kitchen Renovation Contractors: What to Expect, Day by Day</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>kitchen demolition</t>
+          <t>kitchen renovation contractors</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3577,10 +3577,10 @@
         </is>
       </c>
       <c r="G80" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H80" s="6" t="n">
-        <v>48</v>
+        <v>17</v>
+      </c>
+      <c r="H80" s="8" t="n">
+        <v>52</v>
       </c>
     </row>
     <row r="81">
@@ -3591,12 +3591,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>The Right Order of a Kitchen Remodel, Step by Step</t>
+          <t>The Kitchen Remodel Checklist Every Homeowner Should Use</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>order of kitchen remodel</t>
+          <t>kitchen remodel checklist</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
@@ -3606,19 +3606,19 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G81" s="3" t="n">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="H81" s="6" t="n">
-        <v>30</v>
+        <v>38</v>
       </c>
     </row>
     <row r="82">
@@ -3667,12 +3667,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling in Waxhaw, NC: Local Process and Timeline</t>
+          <t>Kitchen Remodeling in Mooresville, NC: A Lake Norman Homeowner's Guide</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>kitchen remodeling waxhaw nc</t>
+          <t>kitchen remodeling mooresville nc</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -3691,7 +3691,7 @@
         </is>
       </c>
       <c r="G83" s="3" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H83" s="4" t="n">
         <v>18</v>
@@ -3705,12 +3705,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Kitchen Remodel in Charlotte, NC: Fixed Pricing, Done in 7 Days</t>
+          <t>Kitchen Remodeling in Gastonia, NC: Costs and What to Expect</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>kitchen remodel charlotte nc</t>
+          <t>kitchen remodeling gastonia nc</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -3729,10 +3729,10 @@
         </is>
       </c>
       <c r="G84" s="3" t="n">
-        <v>390</v>
+        <v>10</v>
       </c>
       <c r="H84" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="85">
@@ -3743,12 +3743,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Kitchen Renovation Charlotte NC: Local Crews, Lifetime Warranty</t>
+          <t>Kitchen Remodeling in Huntersville, NC: Costs, Timelines, and Local Style</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>kitchen renovation charlotte nc</t>
+          <t>kitchen remodeling huntersville nc</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -3767,10 +3767,10 @@
         </is>
       </c>
       <c r="G85" s="3" t="n">
-        <v>170</v>
+        <v>10</v>
       </c>
       <c r="H85" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="86">
@@ -3781,12 +3781,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Kitchen Contractors Charlotte NC: Built Around Your Home and Budget</t>
+          <t>Kitchen Contractors in Charlotte, NC: One Fixed Price, One Crew</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>kitchen contractors charlotte nc</t>
+          <t>kitchen contractor charlotte</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -3805,10 +3805,10 @@
         </is>
       </c>
       <c r="G86" s="3" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="H86" s="4" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="87">
@@ -3819,12 +3819,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling Services Charlotte: Fixed Pricing, Finished in 7 Days</t>
+          <t>Kitchen and Bath Remodeling in Charlotte, NC: One Crew, One Timeline</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>kitchen remodeling services charlotte</t>
+          <t>kitchen and bath remodeling charlotte nc</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -3843,10 +3843,10 @@
         </is>
       </c>
       <c r="G87" s="3" t="n">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="H87" s="4" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="88">
@@ -3857,12 +3857,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Ballantyne Kitchen Remodeling: Premium Results Without the Wait</t>
+          <t>Fast Kitchen Remodel Charlotte: The 7-Day Difference, Explained</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>kitchen remodeling ballantyne</t>
+          <t>fast kitchen remodel charlotte</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -3881,10 +3881,10 @@
         </is>
       </c>
       <c r="G88" s="3" t="n">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="H88" s="4" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="89">
@@ -3933,12 +3933,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling in Belmont, NC: Local Trends and Timelines</t>
+          <t>Full Kitchen Remodels in Charlotte: Everything, One Fixed Price</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>kitchen remodeling belmont nc</t>
+          <t>full kitchen remodel charlotte</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -3957,7 +3957,7 @@
         </is>
       </c>
       <c r="G90" s="3" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H90" s="4" t="n">
         <v>18</v>
@@ -3971,12 +3971,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Custom Kitchen Cabinets in Charlotte: Built for Your Space</t>
+          <t>Kitchen Remodeling in Pineville, NC: A Local Homeowner's Guide</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>custom kitchen cabinets charlotte</t>
+          <t>kitchen remodeling pineville nc</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -3995,10 +3995,10 @@
         </is>
       </c>
       <c r="G91" s="3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H91" s="4" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="92">
@@ -4009,34 +4009,34 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>What Granite Countertops Cost, Installed</t>
+          <t>Kitchen Remodeling in Harrisburg, NC: A Local Renovation Guide</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>cost of granite countertops</t>
-        </is>
-      </c>
-      <c r="D92" s="5" t="inlineStr">
-        <is>
-          <t>Cost &amp; Budget</t>
+          <t>kitchen remodeling harrisburg nc</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Charlotte &amp; Local</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G92" s="3" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="H92" s="4" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="93">
@@ -4047,34 +4047,34 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>What a Small Kitchen Remodel Really Costs</t>
+          <t>Kitchen Remodeling in Mint Hill, NC: A Local Homeowner's Guide</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>average cost of small kitchen remodel</t>
-        </is>
-      </c>
-      <c r="D93" s="5" t="inlineStr">
-        <is>
-          <t>Cost &amp; Budget</t>
+          <t>kitchen remodeling mint hill nc</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>Charlotte &amp; Local</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G93" s="3" t="n">
-        <v>390</v>
+        <v>10</v>
       </c>
       <c r="H93" s="4" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="94">
@@ -4085,34 +4085,34 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>How Much for a Small Kitchen Renovation: What to Weigh First</t>
+          <t>Kitchen and Bath Charlotte NC: A Faster Path to Your Dream Kitchen</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>how much for a small kitchen renovation</t>
-        </is>
-      </c>
-      <c r="D94" s="5" t="inlineStr">
-        <is>
-          <t>Cost &amp; Budget</t>
+          <t>kitchen and bath charlotte nc</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>Charlotte &amp; Local</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G94" s="3" t="n">
-        <v>260</v>
+        <v>10</v>
       </c>
       <c r="H94" s="4" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="95">
@@ -4123,12 +4123,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Inexpensive Kitchen Renovations: A Straight Comparison for Homeowners</t>
+          <t>Quartz Countertop Pricing: What Sets the Range</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>inexpensive kitchen renovations</t>
+          <t>quartz price</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
@@ -4143,14 +4143,14 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G95" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="H95" s="6" t="n">
-        <v>40</v>
+      <c r="H95" s="4" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="96">
@@ -4161,12 +4161,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Cheap Backsplash Ideas: A Plain-English Cost Primer</t>
+          <t>Cost of Kitchen Cabinets: Where the Money Goes, and Where to Save</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>cheap backsplash ideas</t>
+          <t>cost of kitchen cabinets</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -4185,10 +4185,10 @@
         </is>
       </c>
       <c r="G96" s="3" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H96" s="6" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="97">
@@ -4199,12 +4199,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>How Much Are Kitchen Cupboards: Budget, Mid-Range, and High-End</t>
+          <t>Cheap Cabinet Doors Replacement: What Sets the Final Number</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>how much are kitchen cupboards</t>
+          <t>cheap cabinet doors replacement</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
@@ -4219,14 +4219,14 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G97" s="3" t="n">
-        <v>720</v>
+        <v>15</v>
       </c>
       <c r="H97" s="6" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="98">
@@ -4237,12 +4237,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Cost of New Kitchen: What Sets the Final Number</t>
+          <t>What a Kitchen Island Costs to Build In</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>cost of new kitchen</t>
+          <t>kitchen island cost</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
@@ -4261,10 +4261,10 @@
         </is>
       </c>
       <c r="G98" s="3" t="n">
-        <v>390</v>
-      </c>
-      <c r="H98" s="6" t="n">
-        <v>47</v>
+        <v>15</v>
+      </c>
+      <c r="H98" s="4" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="99">
@@ -4275,22 +4275,22 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Choosing Kitchen Cabinets: Styles, Finishes, and What Lasts</t>
+          <t>Small Kitchen Remodels on a Budget: What to Budget Before You Start</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>kitchen cabinets</t>
-        </is>
-      </c>
-      <c r="D99" s="7" t="inlineStr">
-        <is>
-          <t>Design &amp; Materials</t>
+          <t>small kitchen remodels on a budget</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>Cost &amp; Budget</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -4299,10 +4299,10 @@
         </is>
       </c>
       <c r="G99" s="3" t="n">
-        <v>990</v>
-      </c>
-      <c r="H99" s="8" t="n">
-        <v>55</v>
+        <v>260</v>
+      </c>
+      <c r="H99" s="4" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="100">
@@ -4313,12 +4313,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Quartz Countertops: Why They Dominate Modern Kitchens</t>
+          <t>Peel-and-Stick Backsplash: Quick Fix or False Economy?</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>quartz countertops</t>
+          <t>peel and stick backsplash</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
@@ -4337,10 +4337,10 @@
         </is>
       </c>
       <c r="G100" s="3" t="n">
-        <v>543</v>
+        <v>199</v>
       </c>
       <c r="H100" s="4" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="101">
@@ -4351,12 +4351,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Kitchen Countertops Compared: Quartz, Granite, and the Alternatives</t>
+          <t>Kitchen Tile Flooring: A Straight Comparison for Homeowners</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>kitchen countertops</t>
+          <t>kitchen tile flooring</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
@@ -4375,10 +4375,10 @@
         </is>
       </c>
       <c r="G101" s="3" t="n">
-        <v>199</v>
-      </c>
-      <c r="H101" s="6" t="n">
-        <v>48</v>
+        <v>22</v>
+      </c>
+      <c r="H101" s="4" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="102">
@@ -4389,12 +4389,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Small Kitchen Ideas: Making a Compact Space Feel Open</t>
+          <t>Kitchen and Laundry Room Combos: Designing the Two as One Project</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>small kitchen ideas</t>
+          <t>kitchen and laundry room remodel</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
@@ -4409,14 +4409,14 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G102" s="3" t="n">
-        <v>89</v>
-      </c>
-      <c r="H102" s="6" t="n">
         <v>40</v>
+      </c>
+      <c r="H102" s="4" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="103">
@@ -4427,12 +4427,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Kitchen Gadgets: What Designers Pick and Why</t>
+          <t>Butcher Block Countertops: Warm Looks, Real Trade-offs</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>kitchen gadgets</t>
+          <t>butcher block countertops</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
@@ -4451,10 +4451,10 @@
         </is>
       </c>
       <c r="G103" s="3" t="n">
-        <v>59</v>
+        <v>243</v>
       </c>
       <c r="H103" s="6" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="104">
@@ -4465,12 +4465,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Waterfall Islands: The Statement Feature Worth the Splurge</t>
+          <t>Kitchen Backsplash Ideas That Pull a Remodel Together</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>waterfall island</t>
+          <t>kitchen backsplash ideas</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
@@ -4485,11 +4485,11 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G104" s="3" t="n">
-        <v>17</v>
+        <v>109</v>
       </c>
       <c r="H104" s="4" t="n">
         <v>28</v>
@@ -4503,12 +4503,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Kitchen Remodel Before and After: What a Week Can Change</t>
+          <t>Small Kitchen Ideas: Making a Compact Space Feel Open</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>kitchen remodel before and after</t>
+          <t>small kitchen ideas</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
@@ -4527,10 +4527,10 @@
         </is>
       </c>
       <c r="G105" s="3" t="n">
-        <v>590</v>
+        <v>89</v>
       </c>
       <c r="H105" s="6" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
     </row>
     <row r="106">
@@ -4541,12 +4541,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Quartz vs Granite Countertops: Which Wins for Your Kitchen</t>
+          <t>Small Kitchen Island: Ideas That Work in Real Kitchens</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>quartz vs granite</t>
+          <t>small kitchen island</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
@@ -4556,7 +4556,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -4565,10 +4565,10 @@
         </is>
       </c>
       <c r="G106" s="3" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="H106" s="6" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="107">
@@ -4579,12 +4579,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Kitchen Flooring Options Ranked for Durability and Looks</t>
+          <t>Kitchen Cooking Utensils: What Designers Pick and Why</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>kitchen flooring options</t>
+          <t>kitchen cooking utensils</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
@@ -4606,7 +4606,7 @@
         <v>40</v>
       </c>
       <c r="H107" s="6" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="108">
@@ -4617,12 +4617,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Farmhouse Kitchen Ideas That Still Feel Fresh in 2026</t>
+          <t>Kitchen Essentials, Weighed Honestly</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>farmhouse kitchen ideas</t>
+          <t>kitchen essentials</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
@@ -4632,19 +4632,19 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G108" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H108" s="6" t="n">
-        <v>38</v>
+        <v>32</v>
+      </c>
+      <c r="H108" s="8" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="109">
@@ -4655,12 +4655,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Choosing a Kitchen Faucet: Finishes, Features, and Value</t>
+          <t>Open-Concept Kitchens: When Knocking Down a Wall Pays Off</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>kitchen faucet ideas</t>
+          <t>open concept kitchen</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
@@ -4670,19 +4670,19 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G109" s="3" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="H109" s="6" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="110">
@@ -4693,12 +4693,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Cabinet Hardware: The Small Detail That Sets the Tone</t>
+          <t>Kitchen Design Ideas: Layouts, Light, and Lasting Style</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>cabinet hardware ideas</t>
+          <t>kitchen design ideas</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
@@ -4731,12 +4731,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Butler's Pantry Ideas: A Kitchen Upgrade That Adds Real Value</t>
+          <t>Kitchen Cabinet Colors: What's Timeless vs What's Trendy</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>butler pantry ideas</t>
+          <t>kitchen cabinet colors</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
@@ -4751,7 +4751,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G111" s="3" t="n">
@@ -4769,12 +4769,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>White Kitchen Cabinets: Why They Endure, and How to Keep Them Clean</t>
+          <t>Kitchen Trends 2026: Bold Cabinets, Brass, and What to Skip</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>white kitchen cabinets</t>
+          <t>kitchen trends 2026</t>
         </is>
       </c>
       <c r="D112" s="7" t="inlineStr">
@@ -4789,11 +4789,11 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G112" s="3" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="H112" s="6" t="n">
         <v>38</v>
@@ -4807,34 +4807,34 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Finding Local Contractors for a Kitchen Remodel</t>
+          <t>Kitchen Sink Ideas: Materials, Mounts, and the Right Size</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>local contractors for kitchen remodel</t>
-        </is>
-      </c>
-      <c r="D113" s="9" t="inlineStr">
-        <is>
-          <t>Process &amp; Planning</t>
+          <t>kitchen sink ideas</t>
+        </is>
+      </c>
+      <c r="D113" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G113" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H113" s="4" t="n">
-        <v>24</v>
+        <v>40</v>
+      </c>
+      <c r="H113" s="6" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="114">
@@ -4845,22 +4845,22 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Kitchen Bath Contractor: A No-Nonsense Buyer's Guide</t>
+          <t>Kitchen Paint Colors That Flatter Cabinets and Counters</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>kitchen bath contractor</t>
-        </is>
-      </c>
-      <c r="D114" s="9" t="inlineStr">
-        <is>
-          <t>Process &amp; Planning</t>
+          <t>kitchen paint colors</t>
+        </is>
+      </c>
+      <c r="D114" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -4869,10 +4869,10 @@
         </is>
       </c>
       <c r="G114" s="3" t="n">
-        <v>480</v>
+        <v>40</v>
       </c>
       <c r="H114" s="6" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="115">
@@ -4883,22 +4883,22 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>What Separates a Great Kitchen Remodeler From the Rest</t>
+          <t>Kitchen Appliances: Where to Splurge and Where to Save</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>kitchen remodeler</t>
-        </is>
-      </c>
-      <c r="D115" s="9" t="inlineStr">
-        <is>
-          <t>Process &amp; Planning</t>
+          <t>kitchen appliances</t>
+        </is>
+      </c>
+      <c r="D115" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>BoFu</t>
+          <t>MoFu</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -4907,7 +4907,7 @@
         </is>
       </c>
       <c r="G115" s="3" t="n">
-        <v>151</v>
+        <v>40</v>
       </c>
       <c r="H115" s="6" t="n">
         <v>48</v>
@@ -4921,34 +4921,34 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Kitchen Cupboard Plans: What It Takes, Start to Finish</t>
+          <t>Kitchen and Mudroom Combos: A Smarter Family Entryway</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>kitchen cupboard plans</t>
-        </is>
-      </c>
-      <c r="D116" s="9" t="inlineStr">
-        <is>
-          <t>Process &amp; Planning</t>
+          <t>kitchen and mudroom</t>
+        </is>
+      </c>
+      <c r="D116" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G116" s="3" t="n">
-        <v>320</v>
-      </c>
-      <c r="H116" s="4" t="n">
-        <v>13</v>
+        <v>40</v>
+      </c>
+      <c r="H116" s="6" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="117">
@@ -4959,17 +4959,17 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>How to Plan a Kitchen Remodel Before Demo Day</t>
+          <t>White Kitchen Cabinets: Why They Endure, and How to Keep Them Clean</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>how to plan a kitchen remodel</t>
-        </is>
-      </c>
-      <c r="D117" s="9" t="inlineStr">
-        <is>
-          <t>Process &amp; Planning</t>
+          <t>white kitchen cabinets</t>
+        </is>
+      </c>
+      <c r="D117" s="7" t="inlineStr">
+        <is>
+          <t>Design &amp; Materials</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -4979,14 +4979,14 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G117" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H117" s="4" t="n">
-        <v>24</v>
+        <v>10</v>
+      </c>
+      <c r="H117" s="6" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="118">
@@ -4997,12 +4997,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Open Kitchen Plans: How to Pick the Right Pro</t>
+          <t>Kitchen Remodel Contractors Concord: What Separates Great From Cheap</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>open kitchen plans</t>
+          <t>kitchen remodel contractors concord</t>
         </is>
       </c>
       <c r="D118" s="9" t="inlineStr">
@@ -5012,19 +5012,19 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="G118" s="3" t="n">
-        <v>260</v>
+        <v>10</v>
       </c>
       <c r="H118" s="6" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="119">
@@ -5035,12 +5035,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Do You Need a Permit for a Kitchen Remodel in North Carolina?</t>
+          <t>Kitchen Contractors: Done Right the First Time</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>kitchen remodel permits</t>
+          <t>kitchen contractors</t>
         </is>
       </c>
       <c r="D119" s="9" t="inlineStr">
@@ -5050,7 +5050,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>ToFu</t>
+          <t>BoFu</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -5059,10 +5059,10 @@
         </is>
       </c>
       <c r="G119" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H119" s="6" t="n">
-        <v>38</v>
+        <v>15</v>
+      </c>
+      <c r="H119" s="8" t="n">
+        <v>53</v>
       </c>
     </row>
     <row r="120">
@@ -5073,12 +5073,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Questions to Ask a Kitchen Remodel Contractor Before You Sign</t>
+          <t>How to Prepare Your Home for a Kitchen Remodel</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>kitchen remodel contractor questions</t>
+          <t>how to prepare for a kitchen remodel</t>
         </is>
       </c>
       <c r="D120" s="9" t="inlineStr">
@@ -5088,19 +5088,19 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="G120" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H120" s="6" t="n">
-        <v>30</v>
+        <v>10</v>
+      </c>
+      <c r="H120" s="4" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="121">
@@ -5111,12 +5111,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Kitchen Renovation Timeline: Week by Week, What Happens</t>
+          <t>Kitchen Demolition: What Tear-Out Day Actually Involves</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>kitchen renovation timeline</t>
+          <t>kitchen demolition</t>
         </is>
       </c>
       <c r="D121" s="9" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>MoFu</t>
+          <t>ToFu</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -5135,10 +5135,10 @@
         </is>
       </c>
       <c r="G121" s="3" t="n">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="H121" s="6" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -6679,9 +6679,9 @@
       <c r="F8" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="G8" s="11" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -6712,9 +6712,9 @@
       <c r="F9" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="G9" s="11" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -7009,9 +7009,9 @@
       <c r="F18" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="G18" s="11" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -7108,9 +7108,9 @@
       <c r="F21" s="6" t="n">
         <v>48</v>
       </c>
-      <c r="G21" s="11" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -7405,9 +7405,9 @@
       <c r="F30" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="G30" s="11" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -7603,9 +7603,9 @@
       <c r="F36" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="G36" s="11" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -7801,9 +7801,9 @@
       <c r="F42" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G42" s="11" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -8032,9 +8032,9 @@
       <c r="F49" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="G49" s="11" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -8098,9 +8098,9 @@
       <c r="F51" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G51" s="11" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -9154,9 +9154,9 @@
       <c r="F83" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="G83" s="11" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -9187,9 +9187,9 @@
       <c r="F84" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="G84" s="11" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -9715,9 +9715,9 @@
       <c r="F100" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G100" s="11" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -9847,9 +9847,9 @@
       <c r="F104" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G104" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G104" s="11" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -9880,9 +9880,9 @@
       <c r="F105" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G105" s="11" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -9946,9 +9946,9 @@
       <c r="F107" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G107" s="11" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -10177,9 +10177,9 @@
       <c r="F114" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G114" s="11" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -10540,9 +10540,9 @@
       <c r="F125" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G125" s="11" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -10969,9 +10969,9 @@
       <c r="F138" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G138" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G138" s="11" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -11002,9 +11002,9 @@
       <c r="F139" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G139" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G139" s="11" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -11101,9 +11101,9 @@
       <c r="F142" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G142" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G142" s="11" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -11629,9 +11629,9 @@
       <c r="F158" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G158" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G158" s="11" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -11761,9 +11761,9 @@
       <c r="F162" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G162" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G162" s="11" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -13741,9 +13741,9 @@
       <c r="F222" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G222" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G222" s="11" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
7 Day Kitchens: slide 12 + xlsx -> de-duplicated title suffixes
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/7-day-kitchens/keyword-research.xlsx
+++ b/decks/7-day-kitchens/keyword-research.xlsx
@@ -817,7 +817,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Kitchen Design Charlotte NC: The 7-Day Difference, Explained</t>
+          <t>Kitchen Design in Charlotte, NC: From First Sketch to Install</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Kitchen Designers Charlotte: Fixed Pricing, Finished in 7 Days</t>
+          <t>Kitchen Designers in Charlotte: Working With Our In-House Team</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1843,7 +1843,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Kitchen Remodeling in Ballantyne, Charlotte: Fixed-Price, 7 Days</t>
+          <t>Kitchen Remodeling in Ballantyne: A South Charlotte Homeowner's Guide</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Affordable Kitchen Remodel Charlotte NC: Fixed Pricing, Finished in 7 Days</t>
+          <t>Affordable Kitchen Remodels in Charlotte, NC: What's Realistic</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2945,7 +2945,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Kitchen Island with Seating: What Designers Pick and Why</t>
+          <t>Kitchen Islands with Seating: Sizing, Stools, and Clearance</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3287,7 +3287,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Kitchen Cooking Utensils: What Designers Pick and Why</t>
+          <t>Kitchen Cooking Utensils: The Essentials Worth Owning</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">

</xml_diff>